<commit_message>
Factor Registry v5: correlation evidence finality + field metadata + backfill complete
- Schema v5: corr_evidence_note column classifies why evidence is final
  (SELF_NEIGHBORS/SELF_PASS/SELF_FAIL/GATED:/ALREADY_SUBMITTED)
- refresh.py: platform only schedules SELF_CORRELATION when all other
  submission checks pass; failing alphas keep PENDING forever. After a
  2-attempt guard, such factors are marked terminal GATED and leave the
  backfill set (corr verdict stays UNKNOWN, never fabricated)
- mark_corr_evidence_final accepts note parameter; migrations backfill
  existing v4 rows with SELF_NEIGHBORS/SELF_PASS notes
- Report includes correlation evidence coverage section with state breakdown
- All 524 brain-linked factors now have terminal evidence (0 PENDING)
- Field metadata: 109 cached fields across 12 datasets, 84/84=100% coverage
- 955 tests pass (6 new v5 finality tests)
</commit_message>
<xml_diff>
--- a/data/experiments.xlsx
+++ b/data/experiments.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BA462"/>
+  <dimension ref="A1:BA484"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -82422,7 +82422,6 @@
       <c r="AM462" t="n">
         <v>0.0434</v>
       </c>
-      <c r="AN462" t="inlineStr"/>
       <c r="AO462" t="inlineStr">
         <is>
           <t>YES</t>
@@ -82436,11 +82435,9 @@
       <c r="AQ462" t="n">
         <v>0.6866</v>
       </c>
-      <c r="AR462" t="inlineStr"/>
       <c r="AS462" t="b">
         <v>1</v>
       </c>
-      <c r="AT462" t="inlineStr"/>
       <c r="AU462" t="n">
         <v>4</v>
       </c>
@@ -82459,7 +82456,4332 @@
       <c r="AZ462" t="n">
         <v>0.63</v>
       </c>
-      <c r="BA462" t="inlineStr"/>
+    </row>
+    <row r="463">
+      <c r="A463" t="inlineStr">
+        <is>
+          <t>2026-09-14T02:15:00+00:00</t>
+        </is>
+      </c>
+      <c r="B463" t="inlineStr">
+        <is>
+          <t>p38_f6_assets</t>
+        </is>
+      </c>
+      <c r="C463" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="D463" t="inlineStr">
+        <is>
+          <t>INFERIOR</t>
+        </is>
+      </c>
+      <c r="E463" t="inlineStr">
+        <is>
+          <t>group_zscore(winsorize(ts_mean(ts_backfill(assets, 60) / cap, 20), std=3.0), subindustry)</t>
+        </is>
+      </c>
+      <c r="F463" t="inlineStr">
+        <is>
+          <t>fundamental6, pv1</t>
+        </is>
+      </c>
+      <c r="G463" t="inlineStr">
+        <is>
+          <t>assets, cap</t>
+        </is>
+      </c>
+      <c r="H463" t="n">
+        <v>2</v>
+      </c>
+      <c r="I463" t="inlineStr">
+        <is>
+          <t>1NY3ixaAu4It93HMjJBWHxB</t>
+        </is>
+      </c>
+      <c r="J463" t="inlineStr">
+        <is>
+          <t>xAYoWW6b</t>
+        </is>
+      </c>
+      <c r="K463" t="inlineStr">
+        <is>
+          <t>https://platform.worldquantbrain.com/alpha/xAYoWW6b</t>
+        </is>
+      </c>
+      <c r="L463" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="M463" t="inlineStr">
+        <is>
+          <t>TOP3000</t>
+        </is>
+      </c>
+      <c r="N463" t="n">
+        <v>1</v>
+      </c>
+      <c r="O463" t="n">
+        <v>12</v>
+      </c>
+      <c r="P463" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="Q463" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="R463" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="S463" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="T463" t="inlineStr">
+        <is>
+          <t>VERIFY</t>
+        </is>
+      </c>
+      <c r="U463" t="inlineStr">
+        <is>
+          <t>EQUITY</t>
+        </is>
+      </c>
+      <c r="V463" t="inlineStr">
+        <is>
+          <t>FASTEXPR</t>
+        </is>
+      </c>
+      <c r="W463" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="X463" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="Y463" t="n">
+        <v>0.0138</v>
+      </c>
+      <c r="Z463" t="n">
+        <v>0.0887</v>
+      </c>
+      <c r="AA463" t="n">
+        <v>0.1711</v>
+      </c>
+      <c r="AB463" t="n">
+        <v>0.012897</v>
+      </c>
+      <c r="AC463" t="n">
+        <v>4390579</v>
+      </c>
+      <c r="AD463" t="n">
+        <v>20000000</v>
+      </c>
+      <c r="AE463" t="n">
+        <v>1133</v>
+      </c>
+      <c r="AF463" t="n">
+        <v>1883</v>
+      </c>
+      <c r="AG463" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="AH463" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="AI463" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="AJ463" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="AK463" t="n">
+        <v>0.0655</v>
+      </c>
+      <c r="AL463" t="n">
+        <v>0.0124</v>
+      </c>
+      <c r="AM463" t="n">
+        <v>0.1136</v>
+      </c>
+      <c r="AN463" t="inlineStr">
+        <is>
+          <t>LOW_FITNESS=0.72(limit 1.0):FAIL, LOW_SHARPE=0.86(limit 1.25):FAIL</t>
+        </is>
+      </c>
+      <c r="AO463" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="AP463" t="inlineStr">
+        <is>
+          <t>5/8</t>
+        </is>
+      </c>
+      <c r="AR463" t="inlineStr">
+        <is>
+          <t>LOW_GRADE</t>
+        </is>
+      </c>
+      <c r="AS463" t="b">
+        <v>0</v>
+      </c>
+      <c r="AT463" t="inlineStr">
+        <is>
+          <t>Sharpe 0.86 &lt; 1.25; Fitness 0.72 &lt; 1.00</t>
+        </is>
+      </c>
+      <c r="AU463" t="n">
+        <v>3</v>
+      </c>
+      <c r="AV463" t="n">
+        <v>1</v>
+      </c>
+      <c r="AW463" t="n">
+        <v>4</v>
+      </c>
+      <c r="AX463" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="AY463" t="n">
+        <v>0.8990550594930212</v>
+      </c>
+      <c r="AZ463" t="n">
+        <v>-0.2</v>
+      </c>
+    </row>
+    <row r="464">
+      <c r="A464" t="inlineStr">
+        <is>
+          <t>2026-09-14T02:15:04+00:00</t>
+        </is>
+      </c>
+      <c r="B464" t="inlineStr">
+        <is>
+          <t>p38_f6_debt</t>
+        </is>
+      </c>
+      <c r="C464" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="D464" t="inlineStr">
+        <is>
+          <t>INFERIOR</t>
+        </is>
+      </c>
+      <c r="E464" t="inlineStr">
+        <is>
+          <t>group_zscore(winsorize(-ts_mean(ts_backfill(debt, 60) / cap, 20), std=3.0), subindustry)</t>
+        </is>
+      </c>
+      <c r="F464" t="inlineStr">
+        <is>
+          <t>fundamental6, pv1</t>
+        </is>
+      </c>
+      <c r="G464" t="inlineStr">
+        <is>
+          <t>debt, cap</t>
+        </is>
+      </c>
+      <c r="H464" t="n">
+        <v>2</v>
+      </c>
+      <c r="I464" t="inlineStr">
+        <is>
+          <t>D0a7coJ5d2b3SdDMMKFLH</t>
+        </is>
+      </c>
+      <c r="J464" t="inlineStr">
+        <is>
+          <t>RRVoKKLo</t>
+        </is>
+      </c>
+      <c r="K464" t="inlineStr">
+        <is>
+          <t>https://platform.worldquantbrain.com/alpha/RRVoKKLo</t>
+        </is>
+      </c>
+      <c r="L464" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="M464" t="inlineStr">
+        <is>
+          <t>TOP3000</t>
+        </is>
+      </c>
+      <c r="N464" t="n">
+        <v>1</v>
+      </c>
+      <c r="O464" t="n">
+        <v>12</v>
+      </c>
+      <c r="P464" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="Q464" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="R464" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="S464" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="T464" t="inlineStr">
+        <is>
+          <t>VERIFY</t>
+        </is>
+      </c>
+      <c r="U464" t="inlineStr">
+        <is>
+          <t>EQUITY</t>
+        </is>
+      </c>
+      <c r="V464" t="inlineStr">
+        <is>
+          <t>FASTEXPR</t>
+        </is>
+      </c>
+      <c r="W464" t="n">
+        <v>-1.11</v>
+      </c>
+      <c r="X464" t="n">
+        <v>-1.03</v>
+      </c>
+      <c r="Y464" t="n">
+        <v>0.0144</v>
+      </c>
+      <c r="Z464" t="n">
+        <v>-0.1067</v>
+      </c>
+      <c r="AA464" t="n">
+        <v>0.6074000000000001</v>
+      </c>
+      <c r="AB464" t="n">
+        <v>-0.014823</v>
+      </c>
+      <c r="AC464" t="n">
+        <v>-5281672</v>
+      </c>
+      <c r="AD464" t="n">
+        <v>20000000</v>
+      </c>
+      <c r="AE464" t="n">
+        <v>1811</v>
+      </c>
+      <c r="AF464" t="n">
+        <v>977</v>
+      </c>
+      <c r="AG464" t="n">
+        <v>-1.26</v>
+      </c>
+      <c r="AH464" t="n">
+        <v>-1.25</v>
+      </c>
+      <c r="AI464" t="n">
+        <v>-0.46</v>
+      </c>
+      <c r="AJ464" t="n">
+        <v>-0.26</v>
+      </c>
+      <c r="AK464" t="n">
+        <v>-0.0406</v>
+      </c>
+      <c r="AL464" t="n">
+        <v>0.0135</v>
+      </c>
+      <c r="AM464" t="n">
+        <v>0.0902</v>
+      </c>
+      <c r="AN464" t="inlineStr">
+        <is>
+          <t>LOW_FITNESS=-1.03(limit 1.0):FAIL, LOW_SHARPE=-1.11(limit 1.25):FAIL, LOW_SUB_UNIVERSE_SHARPE=-0.64(limit -0.48):FAIL</t>
+        </is>
+      </c>
+      <c r="AO464" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="AP464" t="inlineStr">
+        <is>
+          <t>4/8</t>
+        </is>
+      </c>
+      <c r="AR464" t="inlineStr">
+        <is>
+          <t>LOW_GRADE</t>
+        </is>
+      </c>
+      <c r="AS464" t="b">
+        <v>0</v>
+      </c>
+      <c r="AT464" t="inlineStr">
+        <is>
+          <t>Sharpe -1.11 &lt; 1.25; Fitness -1.03 &lt; 1.00; Positive years 0/4 = 0.0% &lt; 60.0%; Negative-sharpe years 4 &gt; 1</t>
+        </is>
+      </c>
+      <c r="AU464" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV464" t="n">
+        <v>4</v>
+      </c>
+      <c r="AW464" t="n">
+        <v>4</v>
+      </c>
+      <c r="AX464" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY464" t="n">
+        <v>0.619408319823577</v>
+      </c>
+      <c r="AZ464" t="n">
+        <v>-2.23</v>
+      </c>
+    </row>
+    <row r="465">
+      <c r="A465" t="inlineStr">
+        <is>
+          <t>2026-09-14T02:15:21+00:00</t>
+        </is>
+      </c>
+      <c r="B465" t="inlineStr">
+        <is>
+          <t>p38_f6_cflow</t>
+        </is>
+      </c>
+      <c r="C465" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="D465" t="inlineStr">
+        <is>
+          <t>INFERIOR</t>
+        </is>
+      </c>
+      <c r="E465" t="inlineStr">
+        <is>
+          <t>group_zscore(winsorize(ts_mean(ts_backfill(cashflow_op, 60) / cap, 20), std=3.0), subindustry)</t>
+        </is>
+      </c>
+      <c r="F465" t="inlineStr">
+        <is>
+          <t>fundamental6, pv1</t>
+        </is>
+      </c>
+      <c r="G465" t="inlineStr">
+        <is>
+          <t>cashflow_op, cap</t>
+        </is>
+      </c>
+      <c r="H465" t="n">
+        <v>2</v>
+      </c>
+      <c r="I465" t="inlineStr">
+        <is>
+          <t>3Y7UGk9d84GMcwra01NURFy</t>
+        </is>
+      </c>
+      <c r="J465" t="inlineStr">
+        <is>
+          <t>E5vMLLp9</t>
+        </is>
+      </c>
+      <c r="K465" t="inlineStr">
+        <is>
+          <t>https://platform.worldquantbrain.com/alpha/E5vMLLp9</t>
+        </is>
+      </c>
+      <c r="L465" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="M465" t="inlineStr">
+        <is>
+          <t>TOP3000</t>
+        </is>
+      </c>
+      <c r="N465" t="n">
+        <v>1</v>
+      </c>
+      <c r="O465" t="n">
+        <v>12</v>
+      </c>
+      <c r="P465" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="Q465" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="R465" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="S465" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="T465" t="inlineStr">
+        <is>
+          <t>VERIFY</t>
+        </is>
+      </c>
+      <c r="U465" t="inlineStr">
+        <is>
+          <t>EQUITY</t>
+        </is>
+      </c>
+      <c r="V465" t="inlineStr">
+        <is>
+          <t>FASTEXPR</t>
+        </is>
+      </c>
+      <c r="W465" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="X465" t="n">
+        <v>0.63</v>
+      </c>
+      <c r="Y465" t="n">
+        <v>0.0159</v>
+      </c>
+      <c r="Z465" t="n">
+        <v>0.0784</v>
+      </c>
+      <c r="AA465" t="n">
+        <v>0.1724</v>
+      </c>
+      <c r="AB465" t="n">
+        <v>0.009838</v>
+      </c>
+      <c r="AC465" t="n">
+        <v>3879659</v>
+      </c>
+      <c r="AD465" t="n">
+        <v>20000000</v>
+      </c>
+      <c r="AE465" t="n">
+        <v>1386</v>
+      </c>
+      <c r="AF465" t="n">
+        <v>1543</v>
+      </c>
+      <c r="AG465" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="AH465" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="AI465" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="AJ465" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="AK465" t="n">
+        <v>0.065</v>
+      </c>
+      <c r="AL465" t="n">
+        <v>0.0156</v>
+      </c>
+      <c r="AM465" t="n">
+        <v>0.0442</v>
+      </c>
+      <c r="AN465" t="inlineStr">
+        <is>
+          <t>LOW_FITNESS=0.63(limit 1.0):FAIL, LOW_SHARPE=0.8(limit 1.25):FAIL</t>
+        </is>
+      </c>
+      <c r="AO465" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="AP465" t="inlineStr">
+        <is>
+          <t>5/8</t>
+        </is>
+      </c>
+      <c r="AR465" t="inlineStr">
+        <is>
+          <t>LOW_GRADE</t>
+        </is>
+      </c>
+      <c r="AS465" t="b">
+        <v>0</v>
+      </c>
+      <c r="AT465" t="inlineStr">
+        <is>
+          <t>Sharpe 0.80 &lt; 1.25; Fitness 0.63 &lt; 1.00; Positive years 2/4 = 50.0% &lt; 60.0%; Negative-sharpe years 2 &gt; 1</t>
+        </is>
+      </c>
+      <c r="AU465" t="n">
+        <v>2</v>
+      </c>
+      <c r="AV465" t="n">
+        <v>2</v>
+      </c>
+      <c r="AW465" t="n">
+        <v>4</v>
+      </c>
+      <c r="AX465" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AY465" t="n">
+        <v>1.413915956955481</v>
+      </c>
+      <c r="AZ465" t="n">
+        <v>-0.97</v>
+      </c>
+    </row>
+    <row r="466">
+      <c r="A466" t="inlineStr">
+        <is>
+          <t>2026-09-14T02:16:41+00:00</t>
+        </is>
+      </c>
+      <c r="B466" t="inlineStr">
+        <is>
+          <t>p38_f6_bvps</t>
+        </is>
+      </c>
+      <c r="C466" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="D466" t="inlineStr">
+        <is>
+          <t>INFERIOR</t>
+        </is>
+      </c>
+      <c r="E466" t="inlineStr">
+        <is>
+          <t>group_zscore(winsorize(ts_mean(ts_backfill(bookvalue_ps, 60), 20), std=3.0), subindustry)</t>
+        </is>
+      </c>
+      <c r="F466" t="inlineStr">
+        <is>
+          <t>fundamental6</t>
+        </is>
+      </c>
+      <c r="G466" t="inlineStr">
+        <is>
+          <t>bookvalue_ps</t>
+        </is>
+      </c>
+      <c r="H466" t="n">
+        <v>1</v>
+      </c>
+      <c r="I466" t="inlineStr">
+        <is>
+          <t>XYhMaPD5f1c9RQhkbbv66</t>
+        </is>
+      </c>
+      <c r="J466" t="inlineStr">
+        <is>
+          <t>j23JxKpe</t>
+        </is>
+      </c>
+      <c r="K466" t="inlineStr">
+        <is>
+          <t>https://platform.worldquantbrain.com/alpha/j23JxKpe</t>
+        </is>
+      </c>
+      <c r="L466" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="M466" t="inlineStr">
+        <is>
+          <t>TOP3000</t>
+        </is>
+      </c>
+      <c r="N466" t="n">
+        <v>1</v>
+      </c>
+      <c r="O466" t="n">
+        <v>12</v>
+      </c>
+      <c r="P466" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="Q466" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="R466" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="S466" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="T466" t="inlineStr">
+        <is>
+          <t>VERIFY</t>
+        </is>
+      </c>
+      <c r="U466" t="inlineStr">
+        <is>
+          <t>EQUITY</t>
+        </is>
+      </c>
+      <c r="V466" t="inlineStr">
+        <is>
+          <t>FASTEXPR</t>
+        </is>
+      </c>
+      <c r="W466" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="X466" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="Y466" t="n">
+        <v>0.008399999999999999</v>
+      </c>
+      <c r="Z466" t="n">
+        <v>0.0152</v>
+      </c>
+      <c r="AA466" t="n">
+        <v>0.2849</v>
+      </c>
+      <c r="AB466" t="n">
+        <v>0.00361</v>
+      </c>
+      <c r="AC466" t="n">
+        <v>750454</v>
+      </c>
+      <c r="AD466" t="n">
+        <v>20000000</v>
+      </c>
+      <c r="AE466" t="n">
+        <v>1111</v>
+      </c>
+      <c r="AF466" t="n">
+        <v>1795</v>
+      </c>
+      <c r="AG466" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="AH466" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="AI466" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="AJ466" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="AK466" t="n">
+        <v>0.0222</v>
+      </c>
+      <c r="AL466" t="n">
+        <v>0.0062</v>
+      </c>
+      <c r="AM466" t="n">
+        <v>0.06270000000000001</v>
+      </c>
+      <c r="AN466" t="inlineStr">
+        <is>
+          <t>LOW_FITNESS=0.07(limit 1.0):FAIL, LOW_SHARPE=0.19(limit 1.25):FAIL, LOW_SUB_UNIVERSE_SHARPE=-0.1(limit 0.08):FAIL, LOW_TURNOVER=0.0084(limit 0.01):FAIL</t>
+        </is>
+      </c>
+      <c r="AO466" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="AP466" t="inlineStr">
+        <is>
+          <t>3/8</t>
+        </is>
+      </c>
+      <c r="AR466" t="inlineStr">
+        <is>
+          <t>LOW_GRADE</t>
+        </is>
+      </c>
+      <c r="AS466" t="b">
+        <v>0</v>
+      </c>
+      <c r="AT466" t="inlineStr">
+        <is>
+          <t>Sharpe 0.19 &lt; 1.25; Fitness 0.07 &lt; 1.00</t>
+        </is>
+      </c>
+      <c r="AU466" t="n">
+        <v>3</v>
+      </c>
+      <c r="AV466" t="n">
+        <v>1</v>
+      </c>
+      <c r="AW466" t="n">
+        <v>4</v>
+      </c>
+      <c r="AX466" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="AY466" t="n">
+        <v>2.065387372867376</v>
+      </c>
+      <c r="AZ466" t="n">
+        <v>-3.27</v>
+      </c>
+    </row>
+    <row r="467">
+      <c r="A467" t="inlineStr">
+        <is>
+          <t>2026-09-14T02:17:11+00:00</t>
+        </is>
+      </c>
+      <c r="B467" t="inlineStr">
+        <is>
+          <t>p38_f6_capex</t>
+        </is>
+      </c>
+      <c r="C467" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="D467" t="inlineStr">
+        <is>
+          <t>INFERIOR</t>
+        </is>
+      </c>
+      <c r="E467" t="inlineStr">
+        <is>
+          <t>group_zscore(winsorize(ts_mean(ts_backfill(capex, 60) / cap, 20), std=3.0), subindustry)</t>
+        </is>
+      </c>
+      <c r="F467" t="inlineStr">
+        <is>
+          <t>fundamental6, pv1</t>
+        </is>
+      </c>
+      <c r="G467" t="inlineStr">
+        <is>
+          <t>capex, cap</t>
+        </is>
+      </c>
+      <c r="H467" t="n">
+        <v>2</v>
+      </c>
+      <c r="I467" t="inlineStr">
+        <is>
+          <t>1mLEceg6K4COcjdZc55TUQb</t>
+        </is>
+      </c>
+      <c r="J467" t="inlineStr">
+        <is>
+          <t>rK5wVqgJ</t>
+        </is>
+      </c>
+      <c r="K467" t="inlineStr">
+        <is>
+          <t>https://platform.worldquantbrain.com/alpha/rK5wVqgJ</t>
+        </is>
+      </c>
+      <c r="L467" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="M467" t="inlineStr">
+        <is>
+          <t>TOP3000</t>
+        </is>
+      </c>
+      <c r="N467" t="n">
+        <v>1</v>
+      </c>
+      <c r="O467" t="n">
+        <v>12</v>
+      </c>
+      <c r="P467" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="Q467" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="R467" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="S467" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="T467" t="inlineStr">
+        <is>
+          <t>VERIFY</t>
+        </is>
+      </c>
+      <c r="U467" t="inlineStr">
+        <is>
+          <t>EQUITY</t>
+        </is>
+      </c>
+      <c r="V467" t="inlineStr">
+        <is>
+          <t>FASTEXPR</t>
+        </is>
+      </c>
+      <c r="W467" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="X467" t="n">
+        <v>0.8100000000000001</v>
+      </c>
+      <c r="Y467" t="n">
+        <v>0.0131</v>
+      </c>
+      <c r="Z467" t="n">
+        <v>0.0829</v>
+      </c>
+      <c r="AA467" t="n">
+        <v>0.1314</v>
+      </c>
+      <c r="AB467" t="n">
+        <v>0.012698</v>
+      </c>
+      <c r="AC467" t="n">
+        <v>4103063</v>
+      </c>
+      <c r="AD467" t="n">
+        <v>20000000</v>
+      </c>
+      <c r="AE467" t="n">
+        <v>918</v>
+      </c>
+      <c r="AF467" t="n">
+        <v>1907</v>
+      </c>
+      <c r="AG467" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="AH467" t="n">
+        <v>0.8100000000000001</v>
+      </c>
+      <c r="AI467" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ467" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="AK467" t="n">
+        <v>0.07920000000000001</v>
+      </c>
+      <c r="AL467" t="n">
+        <v>0.0114</v>
+      </c>
+      <c r="AM467" t="n">
+        <v>0.0823</v>
+      </c>
+      <c r="AN467" t="inlineStr">
+        <is>
+          <t>LOW_FITNESS=0.81(limit 1.0):FAIL, LOW_SHARPE=0.99(limit 1.25):FAIL</t>
+        </is>
+      </c>
+      <c r="AO467" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="AP467" t="inlineStr">
+        <is>
+          <t>5/8</t>
+        </is>
+      </c>
+      <c r="AR467" t="inlineStr">
+        <is>
+          <t>LOW_GRADE</t>
+        </is>
+      </c>
+      <c r="AS467" t="b">
+        <v>0</v>
+      </c>
+      <c r="AT467" t="inlineStr">
+        <is>
+          <t>Sharpe 0.99 &lt; 1.25; Fitness 0.81 &lt; 1.00</t>
+        </is>
+      </c>
+      <c r="AU467" t="n">
+        <v>3</v>
+      </c>
+      <c r="AV467" t="n">
+        <v>1</v>
+      </c>
+      <c r="AW467" t="n">
+        <v>4</v>
+      </c>
+      <c r="AX467" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="AY467" t="n">
+        <v>1.236513916891624</v>
+      </c>
+      <c r="AZ467" t="n">
+        <v>-0.23</v>
+      </c>
+    </row>
+    <row r="468">
+      <c r="A468" t="inlineStr">
+        <is>
+          <t>2026-09-14T02:17:14+00:00</t>
+        </is>
+      </c>
+      <c r="B468" t="inlineStr">
+        <is>
+          <t>p38_f6_cogs</t>
+        </is>
+      </c>
+      <c r="C468" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="D468" t="inlineStr">
+        <is>
+          <t>INFERIOR</t>
+        </is>
+      </c>
+      <c r="E468" t="inlineStr">
+        <is>
+          <t>group_zscore(winsorize(-ts_mean(ts_backfill(cogs, 60) / cap, 20), std=3.0), subindustry)</t>
+        </is>
+      </c>
+      <c r="F468" t="inlineStr">
+        <is>
+          <t>fundamental6, pv1</t>
+        </is>
+      </c>
+      <c r="G468" t="inlineStr">
+        <is>
+          <t>cogs, cap</t>
+        </is>
+      </c>
+      <c r="H468" t="n">
+        <v>2</v>
+      </c>
+      <c r="I468" t="inlineStr">
+        <is>
+          <t>13ny8FaOc4DT8ZE9NS6coDs</t>
+        </is>
+      </c>
+      <c r="J468" t="inlineStr">
+        <is>
+          <t>kqVMOwld</t>
+        </is>
+      </c>
+      <c r="K468" t="inlineStr">
+        <is>
+          <t>https://platform.worldquantbrain.com/alpha/kqVMOwld</t>
+        </is>
+      </c>
+      <c r="L468" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="M468" t="inlineStr">
+        <is>
+          <t>TOP3000</t>
+        </is>
+      </c>
+      <c r="N468" t="n">
+        <v>1</v>
+      </c>
+      <c r="O468" t="n">
+        <v>12</v>
+      </c>
+      <c r="P468" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="Q468" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="R468" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="S468" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="T468" t="inlineStr">
+        <is>
+          <t>VERIFY</t>
+        </is>
+      </c>
+      <c r="U468" t="inlineStr">
+        <is>
+          <t>EQUITY</t>
+        </is>
+      </c>
+      <c r="V468" t="inlineStr">
+        <is>
+          <t>FASTEXPR</t>
+        </is>
+      </c>
+      <c r="W468" t="n">
+        <v>-1.07</v>
+      </c>
+      <c r="X468" t="n">
+        <v>-0.93</v>
+      </c>
+      <c r="Y468" t="n">
+        <v>0.0144</v>
+      </c>
+      <c r="Z468" t="n">
+        <v>-0.0953</v>
+      </c>
+      <c r="AA468" t="n">
+        <v>0.5760999999999999</v>
+      </c>
+      <c r="AB468" t="n">
+        <v>-0.013216</v>
+      </c>
+      <c r="AC468" t="n">
+        <v>-4713915</v>
+      </c>
+      <c r="AD468" t="n">
+        <v>20000000</v>
+      </c>
+      <c r="AE468" t="n">
+        <v>1981</v>
+      </c>
+      <c r="AF468" t="n">
+        <v>1027</v>
+      </c>
+      <c r="AG468" t="n">
+        <v>-1.06</v>
+      </c>
+      <c r="AH468" t="n">
+        <v>-0.9399999999999999</v>
+      </c>
+      <c r="AI468" t="n">
+        <v>-1.15</v>
+      </c>
+      <c r="AJ468" t="n">
+        <v>-0.95</v>
+      </c>
+      <c r="AK468" t="n">
+        <v>-0.0852</v>
+      </c>
+      <c r="AL468" t="n">
+        <v>0.013</v>
+      </c>
+      <c r="AM468" t="n">
+        <v>0.1079</v>
+      </c>
+      <c r="AN468" t="inlineStr">
+        <is>
+          <t>LOW_FITNESS=-0.93(limit 1.0):FAIL, LOW_SHARPE=-1.07(limit 1.25):FAIL, LOW_SUB_UNIVERSE_SHARPE=-0.49(limit -0.46):FAIL</t>
+        </is>
+      </c>
+      <c r="AO468" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="AP468" t="inlineStr">
+        <is>
+          <t>4/8</t>
+        </is>
+      </c>
+      <c r="AR468" t="inlineStr">
+        <is>
+          <t>LOW_GRADE</t>
+        </is>
+      </c>
+      <c r="AS468" t="b">
+        <v>0</v>
+      </c>
+      <c r="AT468" t="inlineStr">
+        <is>
+          <t>Sharpe -1.07 &lt; 1.25; Fitness -0.93 &lt; 1.00; Positive years 1/4 = 25.0% &lt; 60.0%; Negative-sharpe years 3 &gt; 1</t>
+        </is>
+      </c>
+      <c r="AU468" t="n">
+        <v>1</v>
+      </c>
+      <c r="AV468" t="n">
+        <v>3</v>
+      </c>
+      <c r="AW468" t="n">
+        <v>4</v>
+      </c>
+      <c r="AX468" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="AY468" t="n">
+        <v>1.00619332138511</v>
+      </c>
+      <c r="AZ468" t="n">
+        <v>-2.3</v>
+      </c>
+    </row>
+    <row r="469">
+      <c r="A469" t="inlineStr">
+        <is>
+          <t>2026-09-14T02:18:25+00:00</t>
+        </is>
+      </c>
+      <c r="B469" t="inlineStr">
+        <is>
+          <t>p38_a4_eps</t>
+        </is>
+      </c>
+      <c r="C469" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="D469" t="inlineStr">
+        <is>
+          <t>INFERIOR</t>
+        </is>
+      </c>
+      <c r="E469" t="inlineStr">
+        <is>
+          <t>group_zscore(winsorize(ts_mean(ts_backfill(actual_eps_value_quarterly, 40) / cap, 20), std=3.0), subindustry)</t>
+        </is>
+      </c>
+      <c r="F469" t="inlineStr">
+        <is>
+          <t>analyst4, pv1</t>
+        </is>
+      </c>
+      <c r="G469" t="inlineStr">
+        <is>
+          <t>actual_eps_value_quarterly, cap</t>
+        </is>
+      </c>
+      <c r="H469" t="n">
+        <v>2</v>
+      </c>
+      <c r="I469" t="inlineStr">
+        <is>
+          <t>5SonpdCI4ZIane18nzPtArx</t>
+        </is>
+      </c>
+      <c r="J469" t="inlineStr">
+        <is>
+          <t>LL9w3Pm9</t>
+        </is>
+      </c>
+      <c r="K469" t="inlineStr">
+        <is>
+          <t>https://platform.worldquantbrain.com/alpha/LL9w3Pm9</t>
+        </is>
+      </c>
+      <c r="L469" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="M469" t="inlineStr">
+        <is>
+          <t>TOP3000</t>
+        </is>
+      </c>
+      <c r="N469" t="n">
+        <v>1</v>
+      </c>
+      <c r="O469" t="n">
+        <v>12</v>
+      </c>
+      <c r="P469" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="Q469" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="R469" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="S469" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="T469" t="inlineStr">
+        <is>
+          <t>VERIFY</t>
+        </is>
+      </c>
+      <c r="U469" t="inlineStr">
+        <is>
+          <t>EQUITY</t>
+        </is>
+      </c>
+      <c r="V469" t="inlineStr">
+        <is>
+          <t>FASTEXPR</t>
+        </is>
+      </c>
+      <c r="W469" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="X469" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="Y469" t="n">
+        <v>0.0233</v>
+      </c>
+      <c r="Z469" t="n">
+        <v>0.0416</v>
+      </c>
+      <c r="AA469" t="n">
+        <v>0.2427</v>
+      </c>
+      <c r="AB469" t="n">
+        <v>0.003565</v>
+      </c>
+      <c r="AC469" t="n">
+        <v>2058188</v>
+      </c>
+      <c r="AD469" t="n">
+        <v>20000000</v>
+      </c>
+      <c r="AE469" t="n">
+        <v>1406</v>
+      </c>
+      <c r="AF469" t="n">
+        <v>1593</v>
+      </c>
+      <c r="AG469" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="AH469" t="n">
+        <v>0.47</v>
+      </c>
+      <c r="AI469" t="n">
+        <v>-0.25</v>
+      </c>
+      <c r="AJ469" t="n">
+        <v>-0.1</v>
+      </c>
+      <c r="AK469" t="n">
+        <v>-0.0209</v>
+      </c>
+      <c r="AL469" t="n">
+        <v>0.0211</v>
+      </c>
+      <c r="AM469" t="n">
+        <v>0.0861</v>
+      </c>
+      <c r="AN469" t="inlineStr">
+        <is>
+          <t>LOW_FITNESS=0.29(limit 1.0):FAIL, LOW_SHARPE=0.5(limit 1.25):FAIL, LOW_SUB_UNIVERSE_SHARPE=-0.05(limit 0.22):FAIL</t>
+        </is>
+      </c>
+      <c r="AO469" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="AP469" t="inlineStr">
+        <is>
+          <t>4/8</t>
+        </is>
+      </c>
+      <c r="AR469" t="inlineStr">
+        <is>
+          <t>LOW_GRADE</t>
+        </is>
+      </c>
+      <c r="AS469" t="b">
+        <v>0</v>
+      </c>
+      <c r="AT469" t="inlineStr">
+        <is>
+          <t>Sharpe 0.50 &lt; 1.25; Fitness 0.29 &lt; 1.00; Positive years 2/4 = 50.0% &lt; 60.0%; Negative-sharpe years 2 &gt; 1</t>
+        </is>
+      </c>
+      <c r="AU469" t="n">
+        <v>2</v>
+      </c>
+      <c r="AV469" t="n">
+        <v>2</v>
+      </c>
+      <c r="AW469" t="n">
+        <v>4</v>
+      </c>
+      <c r="AX469" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AY469" t="n">
+        <v>2.775036035802058</v>
+      </c>
+      <c r="AZ469" t="n">
+        <v>-3.4</v>
+      </c>
+    </row>
+    <row r="470">
+      <c r="A470" t="inlineStr">
+        <is>
+          <t>2026-09-14T02:18:42+00:00</t>
+        </is>
+      </c>
+      <c r="B470" t="inlineStr">
+        <is>
+          <t>p38_a4_adjni</t>
+        </is>
+      </c>
+      <c r="C470" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="D470" t="inlineStr">
+        <is>
+          <t>INFERIOR</t>
+        </is>
+      </c>
+      <c r="E470" t="inlineStr">
+        <is>
+          <t>group_zscore(winsorize(ts_mean(ts_backfill(adj_net_income_avg, 40) / cap, 20), std=3.0), subindustry)</t>
+        </is>
+      </c>
+      <c r="F470" t="inlineStr">
+        <is>
+          <t>analyst4, pv1</t>
+        </is>
+      </c>
+      <c r="G470" t="inlineStr">
+        <is>
+          <t>adj_net_income_avg, cap</t>
+        </is>
+      </c>
+      <c r="H470" t="n">
+        <v>2</v>
+      </c>
+      <c r="I470" t="inlineStr">
+        <is>
+          <t>3qOH2AdVo4kEcjiiw6KEvvA</t>
+        </is>
+      </c>
+      <c r="J470" t="inlineStr">
+        <is>
+          <t>ZY09NYd8</t>
+        </is>
+      </c>
+      <c r="K470" t="inlineStr">
+        <is>
+          <t>https://platform.worldquantbrain.com/alpha/ZY09NYd8</t>
+        </is>
+      </c>
+      <c r="L470" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="M470" t="inlineStr">
+        <is>
+          <t>TOP3000</t>
+        </is>
+      </c>
+      <c r="N470" t="n">
+        <v>1</v>
+      </c>
+      <c r="O470" t="n">
+        <v>12</v>
+      </c>
+      <c r="P470" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="Q470" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="R470" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="S470" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="T470" t="inlineStr">
+        <is>
+          <t>VERIFY</t>
+        </is>
+      </c>
+      <c r="U470" t="inlineStr">
+        <is>
+          <t>EQUITY</t>
+        </is>
+      </c>
+      <c r="V470" t="inlineStr">
+        <is>
+          <t>FASTEXPR</t>
+        </is>
+      </c>
+      <c r="W470" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="X470" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="Y470" t="n">
+        <v>0.0173</v>
+      </c>
+      <c r="Z470" t="n">
+        <v>0.0646</v>
+      </c>
+      <c r="AA470" t="n">
+        <v>0.09760000000000001</v>
+      </c>
+      <c r="AB470" t="n">
+        <v>0.007467</v>
+      </c>
+      <c r="AC470" t="n">
+        <v>3194042</v>
+      </c>
+      <c r="AD470" t="n">
+        <v>20000000</v>
+      </c>
+      <c r="AE470" t="n">
+        <v>1194</v>
+      </c>
+      <c r="AF470" t="n">
+        <v>1429</v>
+      </c>
+      <c r="AG470" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="AH470" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="AI470" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="AJ470" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="AK470" t="n">
+        <v>0.0263</v>
+      </c>
+      <c r="AL470" t="n">
+        <v>0.0157</v>
+      </c>
+      <c r="AM470" t="n">
+        <v>0.0593</v>
+      </c>
+      <c r="AN470" t="inlineStr">
+        <is>
+          <t>LOW_FITNESS=0.62(limit 1.0):FAIL, LOW_SHARPE=0.86(limit 1.25):FAIL, LOW_SUB_UNIVERSE_SHARPE=0.29(limit 0.37):FAIL</t>
+        </is>
+      </c>
+      <c r="AO470" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="AP470" t="inlineStr">
+        <is>
+          <t>4/8</t>
+        </is>
+      </c>
+      <c r="AR470" t="inlineStr">
+        <is>
+          <t>LOW_GRADE</t>
+        </is>
+      </c>
+      <c r="AS470" t="b">
+        <v>0</v>
+      </c>
+      <c r="AT470" t="inlineStr">
+        <is>
+          <t>Sharpe 0.86 &lt; 1.25; Fitness 0.62 &lt; 1.00</t>
+        </is>
+      </c>
+      <c r="AU470" t="n">
+        <v>3</v>
+      </c>
+      <c r="AV470" t="n">
+        <v>1</v>
+      </c>
+      <c r="AW470" t="n">
+        <v>4</v>
+      </c>
+      <c r="AX470" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="AY470" t="n">
+        <v>1.299923074647112</v>
+      </c>
+      <c r="AZ470" t="n">
+        <v>-0.63</v>
+      </c>
+    </row>
+    <row r="471">
+      <c r="A471" t="inlineStr">
+        <is>
+          <t>2026-09-14T02:19:04+00:00</t>
+        </is>
+      </c>
+      <c r="B471" t="inlineStr">
+        <is>
+          <t>p38_o9_be180</t>
+        </is>
+      </c>
+      <c r="C471" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="D471" t="inlineStr">
+        <is>
+          <t>INFERIOR</t>
+        </is>
+      </c>
+      <c r="E471" t="inlineStr">
+        <is>
+          <t>group_zscore(winsorize(ts_mean(call_breakeven_180 / close, 20), std=3.0), industry)</t>
+        </is>
+      </c>
+      <c r="F471" t="inlineStr">
+        <is>
+          <t>option9, pv1</t>
+        </is>
+      </c>
+      <c r="G471" t="inlineStr">
+        <is>
+          <t>call_breakeven_180, close</t>
+        </is>
+      </c>
+      <c r="H471" t="n">
+        <v>2</v>
+      </c>
+      <c r="I471" t="inlineStr">
+        <is>
+          <t>4x0tipc2P5eead8dF7lfzMb</t>
+        </is>
+      </c>
+      <c r="J471" t="inlineStr">
+        <is>
+          <t>xAYo5O1n</t>
+        </is>
+      </c>
+      <c r="K471" t="inlineStr">
+        <is>
+          <t>https://platform.worldquantbrain.com/alpha/xAYo5O1n</t>
+        </is>
+      </c>
+      <c r="L471" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="M471" t="inlineStr">
+        <is>
+          <t>TOP3000</t>
+        </is>
+      </c>
+      <c r="N471" t="n">
+        <v>1</v>
+      </c>
+      <c r="O471" t="n">
+        <v>12</v>
+      </c>
+      <c r="P471" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="Q471" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="R471" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="S471" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="T471" t="inlineStr">
+        <is>
+          <t>VERIFY</t>
+        </is>
+      </c>
+      <c r="U471" t="inlineStr">
+        <is>
+          <t>EQUITY</t>
+        </is>
+      </c>
+      <c r="V471" t="inlineStr">
+        <is>
+          <t>FASTEXPR</t>
+        </is>
+      </c>
+      <c r="W471" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="X471" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="Y471" t="n">
+        <v>0.0359</v>
+      </c>
+      <c r="Z471" t="n">
+        <v>0.0149</v>
+      </c>
+      <c r="AA471" t="n">
+        <v>0.7968</v>
+      </c>
+      <c r="AB471" t="n">
+        <v>0.000831</v>
+      </c>
+      <c r="AC471" t="n">
+        <v>738315</v>
+      </c>
+      <c r="AD471" t="n">
+        <v>20000000</v>
+      </c>
+      <c r="AE471" t="n">
+        <v>1131</v>
+      </c>
+      <c r="AF471" t="n">
+        <v>1822</v>
+      </c>
+      <c r="AG471" t="n">
+        <v>-0.01</v>
+      </c>
+      <c r="AH471" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI471" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="AJ471" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="AK471" t="n">
+        <v>0.0859</v>
+      </c>
+      <c r="AL471" t="n">
+        <v>0.0351</v>
+      </c>
+      <c r="AM471" t="n">
+        <v>0.2445</v>
+      </c>
+      <c r="AN471" t="inlineStr">
+        <is>
+          <t>LOW_FITNESS=0.02(limit 1.0):FAIL, LOW_SHARPE=0.07(limit 1.25):FAIL</t>
+        </is>
+      </c>
+      <c r="AO471" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="AP471" t="inlineStr">
+        <is>
+          <t>5/8</t>
+        </is>
+      </c>
+      <c r="AR471" t="inlineStr">
+        <is>
+          <t>LOW_GRADE</t>
+        </is>
+      </c>
+      <c r="AS471" t="b">
+        <v>0</v>
+      </c>
+      <c r="AT471" t="inlineStr">
+        <is>
+          <t>Sharpe 0.07 &lt; 1.25; Fitness 0.02 &lt; 1.00; Positive years 2/4 = 50.0% &lt; 60.0%; Negative-sharpe years 2 &gt; 1</t>
+        </is>
+      </c>
+      <c r="AU471" t="n">
+        <v>2</v>
+      </c>
+      <c r="AV471" t="n">
+        <v>2</v>
+      </c>
+      <c r="AW471" t="n">
+        <v>4</v>
+      </c>
+      <c r="AX471" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AY471" t="n">
+        <v>1.511210883144154</v>
+      </c>
+      <c r="AZ471" t="n">
+        <v>-1.16</v>
+      </c>
+    </row>
+    <row r="472">
+      <c r="A472" t="inlineStr">
+        <is>
+          <t>2026-09-14T02:20:11+00:00</t>
+        </is>
+      </c>
+      <c r="B472" t="inlineStr">
+        <is>
+          <t>p38_o9_fp120</t>
+        </is>
+      </c>
+      <c r="C472" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="D472" t="inlineStr">
+        <is>
+          <t>INFERIOR</t>
+        </is>
+      </c>
+      <c r="E472" t="inlineStr">
+        <is>
+          <t>group_zscore(winsorize(ts_mean(forward_price_120 / close, 20), std=3.0), industry)</t>
+        </is>
+      </c>
+      <c r="F472" t="inlineStr">
+        <is>
+          <t>option9, pv1</t>
+        </is>
+      </c>
+      <c r="G472" t="inlineStr">
+        <is>
+          <t>forward_price_120, close</t>
+        </is>
+      </c>
+      <c r="H472" t="n">
+        <v>2</v>
+      </c>
+      <c r="I472" t="inlineStr">
+        <is>
+          <t>1mZeqL48x5iB8xBBBIUvH02</t>
+        </is>
+      </c>
+      <c r="J472" t="inlineStr">
+        <is>
+          <t>ZY09N3vd</t>
+        </is>
+      </c>
+      <c r="K472" t="inlineStr">
+        <is>
+          <t>https://platform.worldquantbrain.com/alpha/ZY09N3vd</t>
+        </is>
+      </c>
+      <c r="L472" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="M472" t="inlineStr">
+        <is>
+          <t>TOP3000</t>
+        </is>
+      </c>
+      <c r="N472" t="n">
+        <v>1</v>
+      </c>
+      <c r="O472" t="n">
+        <v>12</v>
+      </c>
+      <c r="P472" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="Q472" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="R472" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="S472" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="T472" t="inlineStr">
+        <is>
+          <t>VERIFY</t>
+        </is>
+      </c>
+      <c r="U472" t="inlineStr">
+        <is>
+          <t>EQUITY</t>
+        </is>
+      </c>
+      <c r="V472" t="inlineStr">
+        <is>
+          <t>FASTEXPR</t>
+        </is>
+      </c>
+      <c r="W472" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="X472" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="Y472" t="n">
+        <v>0.0305</v>
+      </c>
+      <c r="Z472" t="n">
+        <v>0.0254</v>
+      </c>
+      <c r="AA472" t="n">
+        <v>0.1196</v>
+      </c>
+      <c r="AB472" t="n">
+        <v>0.001667</v>
+      </c>
+      <c r="AC472" t="n">
+        <v>1258247</v>
+      </c>
+      <c r="AD472" t="n">
+        <v>20000000</v>
+      </c>
+      <c r="AE472" t="n">
+        <v>1114</v>
+      </c>
+      <c r="AF472" t="n">
+        <v>1836</v>
+      </c>
+      <c r="AG472" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="AH472" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="AI472" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="AJ472" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="AK472" t="n">
+        <v>0.0165</v>
+      </c>
+      <c r="AL472" t="n">
+        <v>0.0261</v>
+      </c>
+      <c r="AM472" t="n">
+        <v>0.0882</v>
+      </c>
+      <c r="AN472" t="inlineStr">
+        <is>
+          <t>LOW_FITNESS=0.14(limit 1.0):FAIL, LOW_SHARPE=0.3(limit 1.25):FAIL</t>
+        </is>
+      </c>
+      <c r="AO472" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="AP472" t="inlineStr">
+        <is>
+          <t>5/8</t>
+        </is>
+      </c>
+      <c r="AR472" t="inlineStr">
+        <is>
+          <t>LOW_GRADE</t>
+        </is>
+      </c>
+      <c r="AS472" t="b">
+        <v>0</v>
+      </c>
+      <c r="AT472" t="inlineStr">
+        <is>
+          <t>Sharpe 0.30 &lt; 1.25; Fitness 0.14 &lt; 1.00</t>
+        </is>
+      </c>
+      <c r="AU472" t="n">
+        <v>3</v>
+      </c>
+      <c r="AV472" t="n">
+        <v>1</v>
+      </c>
+      <c r="AW472" t="n">
+        <v>4</v>
+      </c>
+      <c r="AX472" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="AY472" t="n">
+        <v>0.4057914078275521</v>
+      </c>
+      <c r="AZ472" t="n">
+        <v>-0.12</v>
+      </c>
+    </row>
+    <row r="473">
+      <c r="A473" t="inlineStr">
+        <is>
+          <t>2026-09-14T02:20:29+00:00</t>
+        </is>
+      </c>
+      <c r="B473" t="inlineStr">
+        <is>
+          <t>p38_o8_ivc180</t>
+        </is>
+      </c>
+      <c r="C473" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="D473" t="inlineStr">
+        <is>
+          <t>INFERIOR</t>
+        </is>
+      </c>
+      <c r="E473" t="inlineStr">
+        <is>
+          <t>group_zscore(winsorize(-ts_mean(implied_volatility_call_180, 20), std=3.0), industry)</t>
+        </is>
+      </c>
+      <c r="F473" t="inlineStr">
+        <is>
+          <t>option8</t>
+        </is>
+      </c>
+      <c r="G473" t="inlineStr">
+        <is>
+          <t>implied_volatility_call_180</t>
+        </is>
+      </c>
+      <c r="H473" t="n">
+        <v>1</v>
+      </c>
+      <c r="I473" t="inlineStr">
+        <is>
+          <t>2FkL3L2D85jRavxV30AVNTq</t>
+        </is>
+      </c>
+      <c r="J473" t="inlineStr">
+        <is>
+          <t>kqVM92ZK</t>
+        </is>
+      </c>
+      <c r="K473" t="inlineStr">
+        <is>
+          <t>https://platform.worldquantbrain.com/alpha/kqVM92ZK</t>
+        </is>
+      </c>
+      <c r="L473" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="M473" t="inlineStr">
+        <is>
+          <t>TOP3000</t>
+        </is>
+      </c>
+      <c r="N473" t="n">
+        <v>1</v>
+      </c>
+      <c r="O473" t="n">
+        <v>12</v>
+      </c>
+      <c r="P473" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="Q473" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="R473" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="S473" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="T473" t="inlineStr">
+        <is>
+          <t>VERIFY</t>
+        </is>
+      </c>
+      <c r="U473" t="inlineStr">
+        <is>
+          <t>EQUITY</t>
+        </is>
+      </c>
+      <c r="V473" t="inlineStr">
+        <is>
+          <t>FASTEXPR</t>
+        </is>
+      </c>
+      <c r="W473" t="n">
+        <v>-0.01</v>
+      </c>
+      <c r="X473" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y473" t="n">
+        <v>0.0194</v>
+      </c>
+      <c r="Z473" t="n">
+        <v>-0.0021</v>
+      </c>
+      <c r="AA473" t="n">
+        <v>0.8554</v>
+      </c>
+      <c r="AB473" t="n">
+        <v>-0.000217</v>
+      </c>
+      <c r="AC473" t="n">
+        <v>-104305</v>
+      </c>
+      <c r="AD473" t="n">
+        <v>20000000</v>
+      </c>
+      <c r="AE473" t="n">
+        <v>1708</v>
+      </c>
+      <c r="AF473" t="n">
+        <v>1223</v>
+      </c>
+      <c r="AG473" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="AH473" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="AI473" t="n">
+        <v>-0.42</v>
+      </c>
+      <c r="AJ473" t="n">
+        <v>-0.35</v>
+      </c>
+      <c r="AK473" t="n">
+        <v>-0.0866</v>
+      </c>
+      <c r="AL473" t="n">
+        <v>0.0188</v>
+      </c>
+      <c r="AM473" t="n">
+        <v>0.2088</v>
+      </c>
+      <c r="AN473" t="inlineStr">
+        <is>
+          <t>LOW_FITNESS=-0.0(limit 1.0):FAIL, LOW_SHARPE=-0.01(limit 1.25):FAIL, LOW_SUB_UNIVERSE_SHARPE=-0.12(limit -0.0):FAIL</t>
+        </is>
+      </c>
+      <c r="AO473" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="AP473" t="inlineStr">
+        <is>
+          <t>4/8</t>
+        </is>
+      </c>
+      <c r="AR473" t="inlineStr">
+        <is>
+          <t>LOW_GRADE</t>
+        </is>
+      </c>
+      <c r="AS473" t="b">
+        <v>0</v>
+      </c>
+      <c r="AT473" t="inlineStr">
+        <is>
+          <t>Sharpe -0.01 &lt; 1.25; Fitness -0.00 &lt; 1.00</t>
+        </is>
+      </c>
+      <c r="AU473" t="n">
+        <v>3</v>
+      </c>
+      <c r="AV473" t="n">
+        <v>1</v>
+      </c>
+      <c r="AW473" t="n">
+        <v>4</v>
+      </c>
+      <c r="AX473" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="AY473" t="n">
+        <v>1.513370961353054</v>
+      </c>
+      <c r="AZ473" t="n">
+        <v>-2.33</v>
+      </c>
+    </row>
+    <row r="474">
+      <c r="A474" t="inlineStr">
+        <is>
+          <t>2026-09-14T02:20:49+00:00</t>
+        </is>
+      </c>
+      <c r="B474" t="inlineStr">
+        <is>
+          <t>p38_o8_hv120</t>
+        </is>
+      </c>
+      <c r="C474" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="D474" t="inlineStr">
+        <is>
+          <t>INFERIOR</t>
+        </is>
+      </c>
+      <c r="E474" t="inlineStr">
+        <is>
+          <t>group_zscore(winsorize(-ts_mean(historical_volatility_120, 20), std=3.0), industry)</t>
+        </is>
+      </c>
+      <c r="F474" t="inlineStr">
+        <is>
+          <t>option8</t>
+        </is>
+      </c>
+      <c r="G474" t="inlineStr">
+        <is>
+          <t>historical_volatility_120</t>
+        </is>
+      </c>
+      <c r="H474" t="n">
+        <v>1</v>
+      </c>
+      <c r="I474" t="inlineStr">
+        <is>
+          <t>37LYh04cr4OIaFNPU9tRJDr</t>
+        </is>
+      </c>
+      <c r="J474" t="inlineStr">
+        <is>
+          <t>j23JOmnQ</t>
+        </is>
+      </c>
+      <c r="K474" t="inlineStr">
+        <is>
+          <t>https://platform.worldquantbrain.com/alpha/j23JOmnQ</t>
+        </is>
+      </c>
+      <c r="L474" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="M474" t="inlineStr">
+        <is>
+          <t>TOP3000</t>
+        </is>
+      </c>
+      <c r="N474" t="n">
+        <v>1</v>
+      </c>
+      <c r="O474" t="n">
+        <v>12</v>
+      </c>
+      <c r="P474" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="Q474" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="R474" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="S474" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="T474" t="inlineStr">
+        <is>
+          <t>VERIFY</t>
+        </is>
+      </c>
+      <c r="U474" t="inlineStr">
+        <is>
+          <t>EQUITY</t>
+        </is>
+      </c>
+      <c r="V474" t="inlineStr">
+        <is>
+          <t>FASTEXPR</t>
+        </is>
+      </c>
+      <c r="W474" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="X474" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y474" t="n">
+        <v>0.0193</v>
+      </c>
+      <c r="Z474" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="AA474" t="n">
+        <v>0.7933</v>
+      </c>
+      <c r="AB474" t="n">
+        <v>0.000521</v>
+      </c>
+      <c r="AC474" t="n">
+        <v>248610</v>
+      </c>
+      <c r="AD474" t="n">
+        <v>20000000</v>
+      </c>
+      <c r="AE474" t="n">
+        <v>1759</v>
+      </c>
+      <c r="AF474" t="n">
+        <v>1201</v>
+      </c>
+      <c r="AG474" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="AH474" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="AI474" t="n">
+        <v>-0.22</v>
+      </c>
+      <c r="AJ474" t="n">
+        <v>-0.13</v>
+      </c>
+      <c r="AK474" t="n">
+        <v>-0.0432</v>
+      </c>
+      <c r="AL474" t="n">
+        <v>0.0182</v>
+      </c>
+      <c r="AM474" t="n">
+        <v>0.1917</v>
+      </c>
+      <c r="AN474" t="inlineStr">
+        <is>
+          <t>LOW_FITNESS=0.0(limit 1.0):FAIL, LOW_SHARPE=0.02(limit 1.25):FAIL, LOW_SUB_UNIVERSE_SHARPE=-0.02(limit 0.01):FAIL</t>
+        </is>
+      </c>
+      <c r="AO474" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="AP474" t="inlineStr">
+        <is>
+          <t>4/8</t>
+        </is>
+      </c>
+      <c r="AR474" t="inlineStr">
+        <is>
+          <t>LOW_GRADE</t>
+        </is>
+      </c>
+      <c r="AS474" t="b">
+        <v>0</v>
+      </c>
+      <c r="AT474" t="inlineStr">
+        <is>
+          <t>Sharpe 0.02 &lt; 1.25; Fitness 0.00 &lt; 1.00</t>
+        </is>
+      </c>
+      <c r="AU474" t="n">
+        <v>3</v>
+      </c>
+      <c r="AV474" t="n">
+        <v>1</v>
+      </c>
+      <c r="AW474" t="n">
+        <v>4</v>
+      </c>
+      <c r="AX474" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="AY474" t="n">
+        <v>1.359963234797176</v>
+      </c>
+      <c r="AZ474" t="n">
+        <v>-1.99</v>
+      </c>
+    </row>
+    <row r="475">
+      <c r="A475" t="inlineStr">
+        <is>
+          <t>2026-09-14T02:28:36+00:00</t>
+        </is>
+      </c>
+      <c r="B475" t="inlineStr">
+        <is>
+          <t>r39_r3d2u_k250_d7</t>
+        </is>
+      </c>
+      <c r="C475" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="D475" t="inlineStr">
+        <is>
+          <t>EXCELLENT</t>
+        </is>
+      </c>
+      <c r="E475" t="inlineStr">
+        <is>
+          <t>ey = ts_backfill(anl4_ebit_value, 40) / cap; np = ts_backfill(anl4_fs_detail_estimates_advanced_af_nd_netprofit_mean, 40) / cap; s = ey + np; r = group_zscore(winsorize(ts_rank(s, 250), std=3.0), subindustry); d = group_zscore(winsorize(ts_mean(ts_backfill(debt, 60) / cap, 20), std=3.0), subindustry); u = group_zscore(winsorize(ts_mean(rel_num_all, 10), std=3.0), industry); group_zscore(winsorize(r + r + r + d + d + u, std=3.0), industry)</t>
+        </is>
+      </c>
+      <c r="F475" t="inlineStr">
+        <is>
+          <t>analyst4, pv1, fundamental6, pv13</t>
+        </is>
+      </c>
+      <c r="G475" t="inlineStr">
+        <is>
+          <t>anl4_ebit_value, cap, anl4_fs_detail_estimates_advanced_af_nd_netprofit_mean, debt, rel_num_all</t>
+        </is>
+      </c>
+      <c r="H475" t="n">
+        <v>5</v>
+      </c>
+      <c r="I475" t="inlineStr">
+        <is>
+          <t>26QxnsXI4PGceX3gGPhs2W</t>
+        </is>
+      </c>
+      <c r="J475" t="inlineStr">
+        <is>
+          <t>LL9w3KJm</t>
+        </is>
+      </c>
+      <c r="K475" t="inlineStr">
+        <is>
+          <t>https://platform.worldquantbrain.com/alpha/LL9w3KJm</t>
+        </is>
+      </c>
+      <c r="L475" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="M475" t="inlineStr">
+        <is>
+          <t>TOP3000</t>
+        </is>
+      </c>
+      <c r="N475" t="n">
+        <v>1</v>
+      </c>
+      <c r="O475" t="n">
+        <v>7</v>
+      </c>
+      <c r="P475" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="Q475" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="R475" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="S475" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="T475" t="inlineStr">
+        <is>
+          <t>VERIFY</t>
+        </is>
+      </c>
+      <c r="U475" t="inlineStr">
+        <is>
+          <t>EQUITY</t>
+        </is>
+      </c>
+      <c r="V475" t="inlineStr">
+        <is>
+          <t>FASTEXPR</t>
+        </is>
+      </c>
+      <c r="W475" t="n">
+        <v>2.11</v>
+      </c>
+      <c r="X475" t="n">
+        <v>2.23</v>
+      </c>
+      <c r="Y475" t="n">
+        <v>0.06370000000000001</v>
+      </c>
+      <c r="Z475" t="n">
+        <v>0.1401</v>
+      </c>
+      <c r="AA475" t="n">
+        <v>0.0578</v>
+      </c>
+      <c r="AB475" t="n">
+        <v>0.004398</v>
+      </c>
+      <c r="AC475" t="n">
+        <v>6931935</v>
+      </c>
+      <c r="AD475" t="n">
+        <v>20000000</v>
+      </c>
+      <c r="AE475" t="n">
+        <v>1285</v>
+      </c>
+      <c r="AF475" t="n">
+        <v>1289</v>
+      </c>
+      <c r="AG475" t="n">
+        <v>2.35</v>
+      </c>
+      <c r="AH475" t="n">
+        <v>2.71</v>
+      </c>
+      <c r="AI475" t="n">
+        <v>0.8100000000000001</v>
+      </c>
+      <c r="AJ475" t="n">
+        <v>0.43</v>
+      </c>
+      <c r="AK475" t="n">
+        <v>0.0359</v>
+      </c>
+      <c r="AL475" t="n">
+        <v>0.0622</v>
+      </c>
+      <c r="AM475" t="n">
+        <v>0.0473</v>
+      </c>
+      <c r="AO475" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="AP475" t="inlineStr">
+        <is>
+          <t>8/8</t>
+        </is>
+      </c>
+      <c r="AQ475" t="n">
+        <v>0.6536</v>
+      </c>
+      <c r="AS475" t="b">
+        <v>1</v>
+      </c>
+      <c r="AU475" t="n">
+        <v>4</v>
+      </c>
+      <c r="AV475" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW475" t="n">
+        <v>4</v>
+      </c>
+      <c r="AX475" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY475" t="n">
+        <v>1.03512881646038</v>
+      </c>
+      <c r="AZ475" t="n">
+        <v>1.62</v>
+      </c>
+    </row>
+    <row r="476">
+      <c r="A476" t="inlineStr">
+        <is>
+          <t>2026-09-14T02:28:43+00:00</t>
+        </is>
+      </c>
+      <c r="B476" t="inlineStr">
+        <is>
+          <t>r39_r3d2g_k250_d7</t>
+        </is>
+      </c>
+      <c r="C476" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="D476" t="inlineStr">
+        <is>
+          <t>GOOD</t>
+        </is>
+      </c>
+      <c r="E476" t="inlineStr">
+        <is>
+          <t>ey = ts_backfill(anl4_ebit_value, 40) / cap; np = ts_backfill(anl4_fs_detail_estimates_advanced_af_nd_netprofit_mean, 40) / cap; s = ey + np; r = group_zscore(winsorize(ts_rank(s, 250), std=3.0), subindustry); d = group_zscore(winsorize(ts_mean(ts_backfill(debt, 60) / cap, 20), std=3.0), subindustry); g = group_zscore(winsorize(ts_mean(ts_backfill(cogs, 60) / cap, 20), std=3.0), subindustry); group_zscore(winsorize(r + r + r + d + d + g, std=3.0), industry)</t>
+        </is>
+      </c>
+      <c r="F476" t="inlineStr">
+        <is>
+          <t>analyst4, pv1, fundamental6</t>
+        </is>
+      </c>
+      <c r="G476" t="inlineStr">
+        <is>
+          <t>anl4_ebit_value, cap, anl4_fs_detail_estimates_advanced_af_nd_netprofit_mean, debt, cogs</t>
+        </is>
+      </c>
+      <c r="H476" t="n">
+        <v>5</v>
+      </c>
+      <c r="I476" t="inlineStr">
+        <is>
+          <t>1eX0uKgfv5gWass18OYTcSwc</t>
+        </is>
+      </c>
+      <c r="J476" t="inlineStr">
+        <is>
+          <t>gJQ5LavK</t>
+        </is>
+      </c>
+      <c r="K476" t="inlineStr">
+        <is>
+          <t>https://platform.worldquantbrain.com/alpha/gJQ5LavK</t>
+        </is>
+      </c>
+      <c r="L476" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="M476" t="inlineStr">
+        <is>
+          <t>TOP3000</t>
+        </is>
+      </c>
+      <c r="N476" t="n">
+        <v>1</v>
+      </c>
+      <c r="O476" t="n">
+        <v>7</v>
+      </c>
+      <c r="P476" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="Q476" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="R476" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="S476" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="T476" t="inlineStr">
+        <is>
+          <t>VERIFY</t>
+        </is>
+      </c>
+      <c r="U476" t="inlineStr">
+        <is>
+          <t>EQUITY</t>
+        </is>
+      </c>
+      <c r="V476" t="inlineStr">
+        <is>
+          <t>FASTEXPR</t>
+        </is>
+      </c>
+      <c r="W476" t="n">
+        <v>1.85</v>
+      </c>
+      <c r="X476" t="n">
+        <v>2</v>
+      </c>
+      <c r="Y476" t="n">
+        <v>0.0613</v>
+      </c>
+      <c r="Z476" t="n">
+        <v>0.1457</v>
+      </c>
+      <c r="AA476" t="n">
+        <v>0.1039</v>
+      </c>
+      <c r="AB476" t="n">
+        <v>0.00475</v>
+      </c>
+      <c r="AC476" t="n">
+        <v>7208409</v>
+      </c>
+      <c r="AD476" t="n">
+        <v>20000000</v>
+      </c>
+      <c r="AE476" t="n">
+        <v>1263</v>
+      </c>
+      <c r="AF476" t="n">
+        <v>1308</v>
+      </c>
+      <c r="AG476" t="n">
+        <v>2.09</v>
+      </c>
+      <c r="AH476" t="n">
+        <v>2.44</v>
+      </c>
+      <c r="AI476" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="AJ476" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="AK476" t="n">
+        <v>0.0462</v>
+      </c>
+      <c r="AL476" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="AM476" t="n">
+        <v>0.0708</v>
+      </c>
+      <c r="AO476" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="AP476" t="inlineStr">
+        <is>
+          <t>8/8</t>
+        </is>
+      </c>
+      <c r="AQ476" t="n">
+        <v>0.5581</v>
+      </c>
+      <c r="AS476" t="b">
+        <v>1</v>
+      </c>
+      <c r="AU476" t="n">
+        <v>4</v>
+      </c>
+      <c r="AV476" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW476" t="n">
+        <v>4</v>
+      </c>
+      <c r="AX476" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY476" t="n">
+        <v>1.140186388271672</v>
+      </c>
+      <c r="AZ476" t="n">
+        <v>1.02</v>
+      </c>
+    </row>
+    <row r="477">
+      <c r="A477" t="inlineStr">
+        <is>
+          <t>2026-09-14T02:28:18+00:00</t>
+        </is>
+      </c>
+      <c r="B477" t="inlineStr">
+        <is>
+          <t>r39_r3g2u_k250_d7</t>
+        </is>
+      </c>
+      <c r="C477" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="D477" t="inlineStr">
+        <is>
+          <t>EXCELLENT</t>
+        </is>
+      </c>
+      <c r="E477" t="inlineStr">
+        <is>
+          <t>ey = ts_backfill(anl4_ebit_value, 40) / cap; np = ts_backfill(anl4_fs_detail_estimates_advanced_af_nd_netprofit_mean, 40) / cap; s = ey + np; r = group_zscore(winsorize(ts_rank(s, 250), std=3.0), subindustry); g = group_zscore(winsorize(ts_mean(ts_backfill(cogs, 60) / cap, 20), std=3.0), subindustry); u = group_zscore(winsorize(ts_mean(rel_num_all, 10), std=3.0), industry); group_zscore(winsorize(r + r + r + g + g + u, std=3.0), industry)</t>
+        </is>
+      </c>
+      <c r="F477" t="inlineStr">
+        <is>
+          <t>analyst4, pv1, fundamental6, pv13</t>
+        </is>
+      </c>
+      <c r="G477" t="inlineStr">
+        <is>
+          <t>anl4_ebit_value, cap, anl4_fs_detail_estimates_advanced_af_nd_netprofit_mean, cogs, rel_num_all</t>
+        </is>
+      </c>
+      <c r="H477" t="n">
+        <v>5</v>
+      </c>
+      <c r="I477" t="inlineStr">
+        <is>
+          <t>4f0534bF24pi9CaXViUkv4D</t>
+        </is>
+      </c>
+      <c r="J477" t="inlineStr">
+        <is>
+          <t>2rOxeAvJ</t>
+        </is>
+      </c>
+      <c r="K477" t="inlineStr">
+        <is>
+          <t>https://platform.worldquantbrain.com/alpha/2rOxeAvJ</t>
+        </is>
+      </c>
+      <c r="L477" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="M477" t="inlineStr">
+        <is>
+          <t>TOP3000</t>
+        </is>
+      </c>
+      <c r="N477" t="n">
+        <v>1</v>
+      </c>
+      <c r="O477" t="n">
+        <v>7</v>
+      </c>
+      <c r="P477" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="Q477" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="R477" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="S477" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="T477" t="inlineStr">
+        <is>
+          <t>VERIFY</t>
+        </is>
+      </c>
+      <c r="U477" t="inlineStr">
+        <is>
+          <t>EQUITY</t>
+        </is>
+      </c>
+      <c r="V477" t="inlineStr">
+        <is>
+          <t>FASTEXPR</t>
+        </is>
+      </c>
+      <c r="W477" t="n">
+        <v>2.16</v>
+      </c>
+      <c r="X477" t="n">
+        <v>2.26</v>
+      </c>
+      <c r="Y477" t="n">
+        <v>0.0635</v>
+      </c>
+      <c r="Z477" t="n">
+        <v>0.1369</v>
+      </c>
+      <c r="AA477" t="n">
+        <v>0.0771</v>
+      </c>
+      <c r="AB477" t="n">
+        <v>0.004311</v>
+      </c>
+      <c r="AC477" t="n">
+        <v>6772175</v>
+      </c>
+      <c r="AD477" t="n">
+        <v>20000000</v>
+      </c>
+      <c r="AE477" t="n">
+        <v>1383</v>
+      </c>
+      <c r="AF477" t="n">
+        <v>1379</v>
+      </c>
+      <c r="AG477" t="n">
+        <v>2.32</v>
+      </c>
+      <c r="AH477" t="n">
+        <v>2.61</v>
+      </c>
+      <c r="AI477" t="n">
+        <v>1.37</v>
+      </c>
+      <c r="AJ477" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AK477" t="n">
+        <v>0.0544</v>
+      </c>
+      <c r="AL477" t="n">
+        <v>0.0621</v>
+      </c>
+      <c r="AM477" t="n">
+        <v>0.0439</v>
+      </c>
+      <c r="AO477" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="AP477" t="inlineStr">
+        <is>
+          <t>8/8</t>
+        </is>
+      </c>
+      <c r="AQ477" t="n">
+        <v>0.6753</v>
+      </c>
+      <c r="AS477" t="b">
+        <v>1</v>
+      </c>
+      <c r="AU477" t="n">
+        <v>4</v>
+      </c>
+      <c r="AV477" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW477" t="n">
+        <v>4</v>
+      </c>
+      <c r="AX477" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY477" t="n">
+        <v>1.444538565309583</v>
+      </c>
+      <c r="AZ477" t="n">
+        <v>0.97</v>
+      </c>
+    </row>
+    <row r="478">
+      <c r="A478" t="inlineStr">
+        <is>
+          <t>2026-09-14T02:30:07+00:00</t>
+        </is>
+      </c>
+      <c r="B478" t="inlineStr">
+        <is>
+          <t>r39_r4d2u_k250_d7</t>
+        </is>
+      </c>
+      <c r="C478" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="D478" t="inlineStr">
+        <is>
+          <t>EXCELLENT</t>
+        </is>
+      </c>
+      <c r="E478" t="inlineStr">
+        <is>
+          <t>ey = ts_backfill(anl4_ebit_value, 40) / cap; np = ts_backfill(anl4_fs_detail_estimates_advanced_af_nd_netprofit_mean, 40) / cap; s = ey + np; r = group_zscore(winsorize(ts_rank(s, 250), std=3.0), subindustry); d = group_zscore(winsorize(ts_mean(ts_backfill(debt, 60) / cap, 20), std=3.0), subindustry); u = group_zscore(winsorize(ts_mean(rel_num_all, 10), std=3.0), industry); group_zscore(winsorize(r + r + r + r + d + d + u, std=3.0), industry)</t>
+        </is>
+      </c>
+      <c r="F478" t="inlineStr">
+        <is>
+          <t>analyst4, pv1, fundamental6, pv13</t>
+        </is>
+      </c>
+      <c r="G478" t="inlineStr">
+        <is>
+          <t>anl4_ebit_value, cap, anl4_fs_detail_estimates_advanced_af_nd_netprofit_mean, debt, rel_num_all</t>
+        </is>
+      </c>
+      <c r="H478" t="n">
+        <v>5</v>
+      </c>
+      <c r="I478" t="inlineStr">
+        <is>
+          <t>3eH7MQ8KV5k6cpmgXqOgSbl</t>
+        </is>
+      </c>
+      <c r="J478" t="inlineStr">
+        <is>
+          <t>vRkbPGlr</t>
+        </is>
+      </c>
+      <c r="K478" t="inlineStr">
+        <is>
+          <t>https://platform.worldquantbrain.com/alpha/vRkbPGlr</t>
+        </is>
+      </c>
+      <c r="L478" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="M478" t="inlineStr">
+        <is>
+          <t>TOP3000</t>
+        </is>
+      </c>
+      <c r="N478" t="n">
+        <v>1</v>
+      </c>
+      <c r="O478" t="n">
+        <v>7</v>
+      </c>
+      <c r="P478" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="Q478" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="R478" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="S478" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="T478" t="inlineStr">
+        <is>
+          <t>VERIFY</t>
+        </is>
+      </c>
+      <c r="U478" t="inlineStr">
+        <is>
+          <t>EQUITY</t>
+        </is>
+      </c>
+      <c r="V478" t="inlineStr">
+        <is>
+          <t>FASTEXPR</t>
+        </is>
+      </c>
+      <c r="W478" t="n">
+        <v>2.23</v>
+      </c>
+      <c r="X478" t="n">
+        <v>2.32</v>
+      </c>
+      <c r="Y478" t="n">
+        <v>0.0673</v>
+      </c>
+      <c r="Z478" t="n">
+        <v>0.1351</v>
+      </c>
+      <c r="AA478" t="n">
+        <v>0.0523</v>
+      </c>
+      <c r="AB478" t="n">
+        <v>0.004013</v>
+      </c>
+      <c r="AC478" t="n">
+        <v>6685932</v>
+      </c>
+      <c r="AD478" t="n">
+        <v>20000000</v>
+      </c>
+      <c r="AE478" t="n">
+        <v>1303</v>
+      </c>
+      <c r="AF478" t="n">
+        <v>1271</v>
+      </c>
+      <c r="AG478" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="AH478" t="n">
+        <v>2.84</v>
+      </c>
+      <c r="AI478" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="AJ478" t="n">
+        <v>0.39</v>
+      </c>
+      <c r="AK478" t="n">
+        <v>0.031</v>
+      </c>
+      <c r="AL478" t="n">
+        <v>0.0655</v>
+      </c>
+      <c r="AM478" t="n">
+        <v>0.0417</v>
+      </c>
+      <c r="AN478" t="inlineStr">
+        <is>
+          <t>SELF_CORRELATION=0.7076(limit 0.7):FAIL</t>
+        </is>
+      </c>
+      <c r="AO478" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="AP478" t="inlineStr">
+        <is>
+          <t>7/8</t>
+        </is>
+      </c>
+      <c r="AQ478" t="n">
+        <v>0.7076</v>
+      </c>
+      <c r="AR478" t="inlineStr">
+        <is>
+          <t>SELF_CORRELATION_BLOCKED</t>
+        </is>
+      </c>
+      <c r="AS478" t="b">
+        <v>1</v>
+      </c>
+      <c r="AU478" t="n">
+        <v>4</v>
+      </c>
+      <c r="AV478" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW478" t="n">
+        <v>4</v>
+      </c>
+      <c r="AX478" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY478" t="n">
+        <v>1.121695145750395</v>
+      </c>
+      <c r="AZ478" t="n">
+        <v>1.77</v>
+      </c>
+    </row>
+    <row r="479">
+      <c r="A479" t="inlineStr">
+        <is>
+          <t>2026-09-14T02:30:29+00:00</t>
+        </is>
+      </c>
+      <c r="B479" t="inlineStr">
+        <is>
+          <t>r39_r4g2u_k250_d7</t>
+        </is>
+      </c>
+      <c r="C479" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="D479" t="inlineStr">
+        <is>
+          <t>EXCELLENT</t>
+        </is>
+      </c>
+      <c r="E479" t="inlineStr">
+        <is>
+          <t>ey = ts_backfill(anl4_ebit_value, 40) / cap; np = ts_backfill(anl4_fs_detail_estimates_advanced_af_nd_netprofit_mean, 40) / cap; s = ey + np; r = group_zscore(winsorize(ts_rank(s, 250), std=3.0), subindustry); g = group_zscore(winsorize(ts_mean(ts_backfill(cogs, 60) / cap, 20), std=3.0), subindustry); u = group_zscore(winsorize(ts_mean(rel_num_all, 10), std=3.0), industry); group_zscore(winsorize(r + r + r + r + g + g + u, std=3.0), industry)</t>
+        </is>
+      </c>
+      <c r="F479" t="inlineStr">
+        <is>
+          <t>analyst4, pv1, fundamental6, pv13</t>
+        </is>
+      </c>
+      <c r="G479" t="inlineStr">
+        <is>
+          <t>anl4_ebit_value, cap, anl4_fs_detail_estimates_advanced_af_nd_netprofit_mean, cogs, rel_num_all</t>
+        </is>
+      </c>
+      <c r="H479" t="n">
+        <v>5</v>
+      </c>
+      <c r="I479" t="inlineStr">
+        <is>
+          <t>3mi9DG4fv4QZani1flTLECeh</t>
+        </is>
+      </c>
+      <c r="J479" t="inlineStr">
+        <is>
+          <t>d5O6vo1K</t>
+        </is>
+      </c>
+      <c r="K479" t="inlineStr">
+        <is>
+          <t>https://platform.worldquantbrain.com/alpha/d5O6vo1K</t>
+        </is>
+      </c>
+      <c r="L479" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="M479" t="inlineStr">
+        <is>
+          <t>TOP3000</t>
+        </is>
+      </c>
+      <c r="N479" t="n">
+        <v>1</v>
+      </c>
+      <c r="O479" t="n">
+        <v>7</v>
+      </c>
+      <c r="P479" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="Q479" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="R479" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="S479" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="T479" t="inlineStr">
+        <is>
+          <t>VERIFY</t>
+        </is>
+      </c>
+      <c r="U479" t="inlineStr">
+        <is>
+          <t>EQUITY</t>
+        </is>
+      </c>
+      <c r="V479" t="inlineStr">
+        <is>
+          <t>FASTEXPR</t>
+        </is>
+      </c>
+      <c r="W479" t="n">
+        <v>2.28</v>
+      </c>
+      <c r="X479" t="n">
+        <v>2.35</v>
+      </c>
+      <c r="Y479" t="n">
+        <v>0.067</v>
+      </c>
+      <c r="Z479" t="n">
+        <v>0.1324</v>
+      </c>
+      <c r="AA479" t="n">
+        <v>0.0673</v>
+      </c>
+      <c r="AB479" t="n">
+        <v>0.003952</v>
+      </c>
+      <c r="AC479" t="n">
+        <v>6549939</v>
+      </c>
+      <c r="AD479" t="n">
+        <v>20000000</v>
+      </c>
+      <c r="AE479" t="n">
+        <v>1400</v>
+      </c>
+      <c r="AF479" t="n">
+        <v>1362</v>
+      </c>
+      <c r="AG479" t="n">
+        <v>2.47</v>
+      </c>
+      <c r="AH479" t="n">
+        <v>2.74</v>
+      </c>
+      <c r="AI479" t="n">
+        <v>1.29</v>
+      </c>
+      <c r="AJ479" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="AK479" t="n">
+        <v>0.0468</v>
+      </c>
+      <c r="AL479" t="n">
+        <v>0.0653</v>
+      </c>
+      <c r="AM479" t="n">
+        <v>0.0409</v>
+      </c>
+      <c r="AN479" t="inlineStr">
+        <is>
+          <t>SELF_CORRELATION=0.7254(limit 0.7):FAIL</t>
+        </is>
+      </c>
+      <c r="AO479" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="AP479" t="inlineStr">
+        <is>
+          <t>7/8</t>
+        </is>
+      </c>
+      <c r="AQ479" t="n">
+        <v>0.7254</v>
+      </c>
+      <c r="AR479" t="inlineStr">
+        <is>
+          <t>SELF_CORRELATION_BLOCKED</t>
+        </is>
+      </c>
+      <c r="AS479" t="b">
+        <v>1</v>
+      </c>
+      <c r="AU479" t="n">
+        <v>4</v>
+      </c>
+      <c r="AV479" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW479" t="n">
+        <v>4</v>
+      </c>
+      <c r="AX479" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY479" t="n">
+        <v>1.476310152598927</v>
+      </c>
+      <c r="AZ479" t="n">
+        <v>1.15</v>
+      </c>
+    </row>
+    <row r="480">
+      <c r="A480" t="inlineStr">
+        <is>
+          <t>2026-09-14T02:31:02+00:00</t>
+        </is>
+      </c>
+      <c r="B480" t="inlineStr">
+        <is>
+          <t>r39_r4d2g_k250_d7</t>
+        </is>
+      </c>
+      <c r="C480" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="D480" t="inlineStr">
+        <is>
+          <t>EXCELLENT</t>
+        </is>
+      </c>
+      <c r="E480" t="inlineStr">
+        <is>
+          <t>ey = ts_backfill(anl4_ebit_value, 40) / cap; np = ts_backfill(anl4_fs_detail_estimates_advanced_af_nd_netprofit_mean, 40) / cap; s = ey + np; r = group_zscore(winsorize(ts_rank(s, 250), std=3.0), subindustry); d = group_zscore(winsorize(ts_mean(ts_backfill(debt, 60) / cap, 20), std=3.0), subindustry); g = group_zscore(winsorize(ts_mean(ts_backfill(cogs, 60) / cap, 20), std=3.0), subindustry); group_zscore(winsorize(r + r + r + r + d + d + g, std=3.0), industry)</t>
+        </is>
+      </c>
+      <c r="F480" t="inlineStr">
+        <is>
+          <t>analyst4, pv1, fundamental6</t>
+        </is>
+      </c>
+      <c r="G480" t="inlineStr">
+        <is>
+          <t>anl4_ebit_value, cap, anl4_fs_detail_estimates_advanced_af_nd_netprofit_mean, debt, cogs</t>
+        </is>
+      </c>
+      <c r="H480" t="n">
+        <v>5</v>
+      </c>
+      <c r="I480" t="inlineStr">
+        <is>
+          <t>1HZQ9M70C4j893686UJkKUp</t>
+        </is>
+      </c>
+      <c r="J480" t="inlineStr">
+        <is>
+          <t>qMWpVVQj</t>
+        </is>
+      </c>
+      <c r="K480" t="inlineStr">
+        <is>
+          <t>https://platform.worldquantbrain.com/alpha/qMWpVVQj</t>
+        </is>
+      </c>
+      <c r="L480" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="M480" t="inlineStr">
+        <is>
+          <t>TOP3000</t>
+        </is>
+      </c>
+      <c r="N480" t="n">
+        <v>1</v>
+      </c>
+      <c r="O480" t="n">
+        <v>7</v>
+      </c>
+      <c r="P480" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="Q480" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="R480" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="S480" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="T480" t="inlineStr">
+        <is>
+          <t>VERIFY</t>
+        </is>
+      </c>
+      <c r="U480" t="inlineStr">
+        <is>
+          <t>EQUITY</t>
+        </is>
+      </c>
+      <c r="V480" t="inlineStr">
+        <is>
+          <t>FASTEXPR</t>
+        </is>
+      </c>
+      <c r="W480" t="n">
+        <v>1.98</v>
+      </c>
+      <c r="X480" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="Y480" t="n">
+        <v>0.0655</v>
+      </c>
+      <c r="Z480" t="n">
+        <v>0.1409</v>
+      </c>
+      <c r="AA480" t="n">
+        <v>0.09030000000000001</v>
+      </c>
+      <c r="AB480" t="n">
+        <v>0.004301</v>
+      </c>
+      <c r="AC480" t="n">
+        <v>6970734</v>
+      </c>
+      <c r="AD480" t="n">
+        <v>20000000</v>
+      </c>
+      <c r="AE480" t="n">
+        <v>1288</v>
+      </c>
+      <c r="AF480" t="n">
+        <v>1284</v>
+      </c>
+      <c r="AG480" t="n">
+        <v>2.24</v>
+      </c>
+      <c r="AH480" t="n">
+        <v>2.58</v>
+      </c>
+      <c r="AI480" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="AJ480" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="AK480" t="n">
+        <v>0.0407</v>
+      </c>
+      <c r="AL480" t="n">
+        <v>0.0639</v>
+      </c>
+      <c r="AM480" t="n">
+        <v>0.0604</v>
+      </c>
+      <c r="AO480" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="AP480" t="inlineStr">
+        <is>
+          <t>8/8</t>
+        </is>
+      </c>
+      <c r="AQ480" t="n">
+        <v>0.6155</v>
+      </c>
+      <c r="AS480" t="b">
+        <v>1</v>
+      </c>
+      <c r="AU480" t="n">
+        <v>4</v>
+      </c>
+      <c r="AV480" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW480" t="n">
+        <v>4</v>
+      </c>
+      <c r="AX480" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY480" t="n">
+        <v>1.172358733494147</v>
+      </c>
+      <c r="AZ480" t="n">
+        <v>1.17</v>
+      </c>
+    </row>
+    <row r="481">
+      <c r="A481" t="inlineStr">
+        <is>
+          <t>2026-09-14T02:32:08+00:00</t>
+        </is>
+      </c>
+      <c r="B481" t="inlineStr">
+        <is>
+          <t>r39_r3d2gu_k250_d7</t>
+        </is>
+      </c>
+      <c r="C481" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="D481" t="inlineStr">
+        <is>
+          <t>EXCELLENT</t>
+        </is>
+      </c>
+      <c r="E481" t="inlineStr">
+        <is>
+          <t>ey = ts_backfill(anl4_ebit_value, 40) / cap; np = ts_backfill(anl4_fs_detail_estimates_advanced_af_nd_netprofit_mean, 40) / cap; s = ey + np; r = group_zscore(winsorize(ts_rank(s, 250), std=3.0), subindustry); d = group_zscore(winsorize(ts_mean(ts_backfill(debt, 60) / cap, 20), std=3.0), subindustry); g = group_zscore(winsorize(ts_mean(ts_backfill(cogs, 60) / cap, 20), std=3.0), subindustry); u = group_zscore(winsorize(ts_mean(rel_num_all, 10), std=3.0), industry); group_zscore(winsorize(r + r + r + d + d + g + u, std=3.0), industry)</t>
+        </is>
+      </c>
+      <c r="F481" t="inlineStr">
+        <is>
+          <t>analyst4, pv1, fundamental6, pv13</t>
+        </is>
+      </c>
+      <c r="G481" t="inlineStr">
+        <is>
+          <t>anl4_ebit_value, cap, anl4_fs_detail_estimates_advanced_af_nd_netprofit_mean, debt, cogs, rel_num_all</t>
+        </is>
+      </c>
+      <c r="H481" t="n">
+        <v>6</v>
+      </c>
+      <c r="I481" t="inlineStr">
+        <is>
+          <t>270GftH65k78OM132jeZKu0</t>
+        </is>
+      </c>
+      <c r="J481" t="inlineStr">
+        <is>
+          <t>XgWxMZg1</t>
+        </is>
+      </c>
+      <c r="K481" t="inlineStr">
+        <is>
+          <t>https://platform.worldquantbrain.com/alpha/XgWxMZg1</t>
+        </is>
+      </c>
+      <c r="L481" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="M481" t="inlineStr">
+        <is>
+          <t>TOP3000</t>
+        </is>
+      </c>
+      <c r="N481" t="n">
+        <v>1</v>
+      </c>
+      <c r="O481" t="n">
+        <v>7</v>
+      </c>
+      <c r="P481" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="Q481" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="R481" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="S481" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="T481" t="inlineStr">
+        <is>
+          <t>VERIFY</t>
+        </is>
+      </c>
+      <c r="U481" t="inlineStr">
+        <is>
+          <t>EQUITY</t>
+        </is>
+      </c>
+      <c r="V481" t="inlineStr">
+        <is>
+          <t>FASTEXPR</t>
+        </is>
+      </c>
+      <c r="W481" t="n">
+        <v>1.96</v>
+      </c>
+      <c r="X481" t="n">
+        <v>2.14</v>
+      </c>
+      <c r="Y481" t="n">
+        <v>0.0594</v>
+      </c>
+      <c r="Z481" t="n">
+        <v>0.1495</v>
+      </c>
+      <c r="AA481" t="n">
+        <v>0.0863</v>
+      </c>
+      <c r="AB481" t="n">
+        <v>0.00503</v>
+      </c>
+      <c r="AC481" t="n">
+        <v>7398221</v>
+      </c>
+      <c r="AD481" t="n">
+        <v>20000000</v>
+      </c>
+      <c r="AE481" t="n">
+        <v>1254</v>
+      </c>
+      <c r="AF481" t="n">
+        <v>1318</v>
+      </c>
+      <c r="AG481" t="n">
+        <v>2.16</v>
+      </c>
+      <c r="AH481" t="n">
+        <v>2.56</v>
+      </c>
+      <c r="AI481" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AJ481" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="AK481" t="n">
+        <v>0.0484</v>
+      </c>
+      <c r="AL481" t="n">
+        <v>0.0583</v>
+      </c>
+      <c r="AM481" t="n">
+        <v>0.0603</v>
+      </c>
+      <c r="AO481" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="AP481" t="inlineStr">
+        <is>
+          <t>8/8</t>
+        </is>
+      </c>
+      <c r="AQ481" t="n">
+        <v>0.5887</v>
+      </c>
+      <c r="AS481" t="b">
+        <v>1</v>
+      </c>
+      <c r="AU481" t="n">
+        <v>4</v>
+      </c>
+      <c r="AV481" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW481" t="n">
+        <v>4</v>
+      </c>
+      <c r="AX481" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY481" t="n">
+        <v>1.130998821101655</v>
+      </c>
+      <c r="AZ481" t="n">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="482">
+      <c r="A482" t="inlineStr">
+        <is>
+          <t>2026-09-14T02:32:57+00:00</t>
+        </is>
+      </c>
+      <c r="B482" t="inlineStr">
+        <is>
+          <t>r39_r4d2gu_k250_d7</t>
+        </is>
+      </c>
+      <c r="C482" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="D482" t="inlineStr">
+        <is>
+          <t>EXCELLENT</t>
+        </is>
+      </c>
+      <c r="E482" t="inlineStr">
+        <is>
+          <t>ey = ts_backfill(anl4_ebit_value, 40) / cap; np = ts_backfill(anl4_fs_detail_estimates_advanced_af_nd_netprofit_mean, 40) / cap; s = ey + np; r = group_zscore(winsorize(ts_rank(s, 250), std=3.0), subindustry); d = group_zscore(winsorize(ts_mean(ts_backfill(debt, 60) / cap, 20), std=3.0), subindustry); g = group_zscore(winsorize(ts_mean(ts_backfill(cogs, 60) / cap, 20), std=3.0), subindustry); u = group_zscore(winsorize(ts_mean(rel_num_all, 10), std=3.0), industry); group_zscore(winsorize(r + r + r + r + d + d + g + u, std=3.0), industry)</t>
+        </is>
+      </c>
+      <c r="F482" t="inlineStr">
+        <is>
+          <t>analyst4, pv1, fundamental6, pv13</t>
+        </is>
+      </c>
+      <c r="G482" t="inlineStr">
+        <is>
+          <t>anl4_ebit_value, cap, anl4_fs_detail_estimates_advanced_af_nd_netprofit_mean, debt, cogs, rel_num_all</t>
+        </is>
+      </c>
+      <c r="H482" t="n">
+        <v>6</v>
+      </c>
+      <c r="I482" t="inlineStr">
+        <is>
+          <t>2r40Xd3t4tA8JNS8vge3QK</t>
+        </is>
+      </c>
+      <c r="J482" t="inlineStr">
+        <is>
+          <t>WjPRJ53N</t>
+        </is>
+      </c>
+      <c r="K482" t="inlineStr">
+        <is>
+          <t>https://platform.worldquantbrain.com/alpha/WjPRJ53N</t>
+        </is>
+      </c>
+      <c r="L482" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="M482" t="inlineStr">
+        <is>
+          <t>TOP3000</t>
+        </is>
+      </c>
+      <c r="N482" t="n">
+        <v>1</v>
+      </c>
+      <c r="O482" t="n">
+        <v>7</v>
+      </c>
+      <c r="P482" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="Q482" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="R482" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="S482" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="T482" t="inlineStr">
+        <is>
+          <t>VERIFY</t>
+        </is>
+      </c>
+      <c r="U482" t="inlineStr">
+        <is>
+          <t>EQUITY</t>
+        </is>
+      </c>
+      <c r="V482" t="inlineStr">
+        <is>
+          <t>FASTEXPR</t>
+        </is>
+      </c>
+      <c r="W482" t="n">
+        <v>2.09</v>
+      </c>
+      <c r="X482" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="Y482" t="n">
+        <v>0.0644</v>
+      </c>
+      <c r="Z482" t="n">
+        <v>0.1454</v>
+      </c>
+      <c r="AA482" t="n">
+        <v>0.07679999999999999</v>
+      </c>
+      <c r="AB482" t="n">
+        <v>0.004514</v>
+      </c>
+      <c r="AC482" t="n">
+        <v>7192716</v>
+      </c>
+      <c r="AD482" t="n">
+        <v>20000000</v>
+      </c>
+      <c r="AE482" t="n">
+        <v>1285</v>
+      </c>
+      <c r="AF482" t="n">
+        <v>1286</v>
+      </c>
+      <c r="AG482" t="n">
+        <v>2.32</v>
+      </c>
+      <c r="AH482" t="n">
+        <v>2.72</v>
+      </c>
+      <c r="AI482" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="AJ482" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="AK482" t="n">
+        <v>0.0425</v>
+      </c>
+      <c r="AL482" t="n">
+        <v>0.0631</v>
+      </c>
+      <c r="AM482" t="n">
+        <v>0.0528</v>
+      </c>
+      <c r="AO482" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="AP482" t="inlineStr">
+        <is>
+          <t>8/8</t>
+        </is>
+      </c>
+      <c r="AQ482" t="n">
+        <v>0.6446</v>
+      </c>
+      <c r="AS482" t="b">
+        <v>1</v>
+      </c>
+      <c r="AU482" t="n">
+        <v>4</v>
+      </c>
+      <c r="AV482" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW482" t="n">
+        <v>4</v>
+      </c>
+      <c r="AX482" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY482" t="n">
+        <v>1.197900941925778</v>
+      </c>
+      <c r="AZ482" t="n">
+        <v>1.34</v>
+      </c>
+    </row>
+    <row r="483">
+      <c r="A483" t="inlineStr">
+        <is>
+          <t>2026-09-14T02:32:52+00:00</t>
+        </is>
+      </c>
+      <c r="B483" t="inlineStr">
+        <is>
+          <t>r39_r3d2g_k500_d7</t>
+        </is>
+      </c>
+      <c r="C483" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="D483" t="inlineStr">
+        <is>
+          <t>GOOD</t>
+        </is>
+      </c>
+      <c r="E483" t="inlineStr">
+        <is>
+          <t>ey = ts_backfill(anl4_ebit_value, 40) / cap; np = ts_backfill(anl4_fs_detail_estimates_advanced_af_nd_netprofit_mean, 40) / cap; s = ey + np; r = group_zscore(winsorize(ts_rank(s, 500), std=3.0), subindustry); d = group_zscore(winsorize(ts_mean(ts_backfill(debt, 60) / cap, 20), std=3.0), subindustry); g = group_zscore(winsorize(ts_mean(ts_backfill(cogs, 60) / cap, 20), std=3.0), subindustry); group_zscore(winsorize(r + r + r + d + d + g, std=3.0), industry)</t>
+        </is>
+      </c>
+      <c r="F483" t="inlineStr">
+        <is>
+          <t>analyst4, pv1, fundamental6</t>
+        </is>
+      </c>
+      <c r="G483" t="inlineStr">
+        <is>
+          <t>anl4_ebit_value, cap, anl4_fs_detail_estimates_advanced_af_nd_netprofit_mean, debt, cogs</t>
+        </is>
+      </c>
+      <c r="H483" t="n">
+        <v>5</v>
+      </c>
+      <c r="I483" t="inlineStr">
+        <is>
+          <t>3WXMqLgoz4qO9Jzsix4Fifc</t>
+        </is>
+      </c>
+      <c r="J483" t="inlineStr">
+        <is>
+          <t>883ZXw9m</t>
+        </is>
+      </c>
+      <c r="K483" t="inlineStr">
+        <is>
+          <t>https://platform.worldquantbrain.com/alpha/883ZXw9m</t>
+        </is>
+      </c>
+      <c r="L483" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="M483" t="inlineStr">
+        <is>
+          <t>TOP3000</t>
+        </is>
+      </c>
+      <c r="N483" t="n">
+        <v>1</v>
+      </c>
+      <c r="O483" t="n">
+        <v>7</v>
+      </c>
+      <c r="P483" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="Q483" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="R483" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="S483" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="T483" t="inlineStr">
+        <is>
+          <t>VERIFY</t>
+        </is>
+      </c>
+      <c r="U483" t="inlineStr">
+        <is>
+          <t>EQUITY</t>
+        </is>
+      </c>
+      <c r="V483" t="inlineStr">
+        <is>
+          <t>FASTEXPR</t>
+        </is>
+      </c>
+      <c r="W483" t="n">
+        <v>1.77</v>
+      </c>
+      <c r="X483" t="n">
+        <v>1.87</v>
+      </c>
+      <c r="Y483" t="n">
+        <v>0.051</v>
+      </c>
+      <c r="Z483" t="n">
+        <v>0.1398</v>
+      </c>
+      <c r="AA483" t="n">
+        <v>0.108</v>
+      </c>
+      <c r="AB483" t="n">
+        <v>0.005478</v>
+      </c>
+      <c r="AC483" t="n">
+        <v>6917154</v>
+      </c>
+      <c r="AD483" t="n">
+        <v>20000000</v>
+      </c>
+      <c r="AE483" t="n">
+        <v>1266</v>
+      </c>
+      <c r="AF483" t="n">
+        <v>1306</v>
+      </c>
+      <c r="AG483" t="n">
+        <v>1.95</v>
+      </c>
+      <c r="AH483" t="n">
+        <v>2.22</v>
+      </c>
+      <c r="AI483" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="AJ483" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="AK483" t="n">
+        <v>0.0546</v>
+      </c>
+      <c r="AL483" t="n">
+        <v>0.0494</v>
+      </c>
+      <c r="AM483" t="n">
+        <v>0.0603</v>
+      </c>
+      <c r="AO483" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="AP483" t="inlineStr">
+        <is>
+          <t>8/8</t>
+        </is>
+      </c>
+      <c r="AQ483" t="n">
+        <v>0.5274</v>
+      </c>
+      <c r="AS483" t="b">
+        <v>1</v>
+      </c>
+      <c r="AU483" t="n">
+        <v>4</v>
+      </c>
+      <c r="AV483" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW483" t="n">
+        <v>4</v>
+      </c>
+      <c r="AX483" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY483" t="n">
+        <v>1.177398261705302</v>
+      </c>
+      <c r="AZ483" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+    </row>
+    <row r="484">
+      <c r="A484" t="inlineStr">
+        <is>
+          <t>2026-09-14T02:33:41+00:00</t>
+        </is>
+      </c>
+      <c r="B484" t="inlineStr">
+        <is>
+          <t>r39_r3d2xu_k250_d7</t>
+        </is>
+      </c>
+      <c r="C484" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="D484" t="inlineStr">
+        <is>
+          <t>EXCELLENT</t>
+        </is>
+      </c>
+      <c r="E484" t="inlineStr">
+        <is>
+          <t>ey = ts_backfill(anl4_ebit_value, 40) / cap; np = ts_backfill(anl4_fs_detail_estimates_advanced_af_nd_netprofit_mean, 40) / cap; s = ey + np; r = group_zscore(winsorize(ts_rank(s, 250), std=3.0), subindustry); d = group_zscore(winsorize(ts_mean(ts_backfill(debt, 60) / cap, 20), std=3.0), subindustry); x = group_zscore(winsorize(ts_mean(ts_backfill(capex, 60) / cap, 20), std=3.0), subindustry); u = group_zscore(winsorize(ts_mean(rel_num_all, 10), std=3.0), industry); group_zscore(winsorize(r + r + r + d + d + x + u, std=3.0), industry)</t>
+        </is>
+      </c>
+      <c r="F484" t="inlineStr">
+        <is>
+          <t>analyst4, pv1, fundamental6, pv13</t>
+        </is>
+      </c>
+      <c r="G484" t="inlineStr">
+        <is>
+          <t>anl4_ebit_value, cap, anl4_fs_detail_estimates_advanced_af_nd_netprofit_mean, debt, capex, rel_num_all</t>
+        </is>
+      </c>
+      <c r="H484" t="n">
+        <v>6</v>
+      </c>
+      <c r="I484" t="inlineStr">
+        <is>
+          <t>4ApirH2Rw4V68Hg56L0IHBT</t>
+        </is>
+      </c>
+      <c r="J484" t="inlineStr">
+        <is>
+          <t>9qV32zMq</t>
+        </is>
+      </c>
+      <c r="K484" t="inlineStr">
+        <is>
+          <t>https://platform.worldquantbrain.com/alpha/9qV32zMq</t>
+        </is>
+      </c>
+      <c r="L484" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="M484" t="inlineStr">
+        <is>
+          <t>TOP3000</t>
+        </is>
+      </c>
+      <c r="N484" t="n">
+        <v>1</v>
+      </c>
+      <c r="O484" t="n">
+        <v>7</v>
+      </c>
+      <c r="P484" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="Q484" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="R484" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="S484" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="T484" t="inlineStr">
+        <is>
+          <t>VERIFY</t>
+        </is>
+      </c>
+      <c r="U484" t="inlineStr">
+        <is>
+          <t>EQUITY</t>
+        </is>
+      </c>
+      <c r="V484" t="inlineStr">
+        <is>
+          <t>FASTEXPR</t>
+        </is>
+      </c>
+      <c r="W484" t="n">
+        <v>1.94</v>
+      </c>
+      <c r="X484" t="n">
+        <v>2.09</v>
+      </c>
+      <c r="Y484" t="n">
+        <v>0.0593</v>
+      </c>
+      <c r="Z484" t="n">
+        <v>0.1448</v>
+      </c>
+      <c r="AA484" t="n">
+        <v>0.0814</v>
+      </c>
+      <c r="AB484" t="n">
+        <v>0.004888</v>
+      </c>
+      <c r="AC484" t="n">
+        <v>7166077</v>
+      </c>
+      <c r="AD484" t="n">
+        <v>20000000</v>
+      </c>
+      <c r="AE484" t="n">
+        <v>1211</v>
+      </c>
+      <c r="AF484" t="n">
+        <v>1267</v>
+      </c>
+      <c r="AG484" t="n">
+        <v>2.15</v>
+      </c>
+      <c r="AH484" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="AI484" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="AJ484" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="AK484" t="n">
+        <v>0.0495</v>
+      </c>
+      <c r="AL484" t="n">
+        <v>0.0584</v>
+      </c>
+      <c r="AM484" t="n">
+        <v>0.0516</v>
+      </c>
+      <c r="AN484" t="inlineStr"/>
+      <c r="AO484" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="AP484" t="inlineStr">
+        <is>
+          <t>8/8</t>
+        </is>
+      </c>
+      <c r="AQ484" t="n">
+        <v>0.5790999999999999</v>
+      </c>
+      <c r="AR484" t="inlineStr"/>
+      <c r="AS484" t="b">
+        <v>1</v>
+      </c>
+      <c r="AT484" t="inlineStr"/>
+      <c r="AU484" t="n">
+        <v>4</v>
+      </c>
+      <c r="AV484" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW484" t="n">
+        <v>4</v>
+      </c>
+      <c r="AX484" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY484" t="n">
+        <v>1.083297435302666</v>
+      </c>
+      <c r="AZ484" t="n">
+        <v>1.27</v>
+      </c>
+      <c r="BA484" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>